<commit_message>
convert latency report values to numbers
</commit_message>
<xml_diff>
--- a/outputs/019ffa1d-1429-7a22-873b-6bcd9dea9c5a/AICO_Agent调用时延报告.xlsx
+++ b/outputs/019ffa1d-1429-7a22-873b-6bcd9dea9c5a/AICO_Agent调用时延报告.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R471278ed864046c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="调用明细" sheetId="2" r:id="R6efd1cab6a584346"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="3" r:id="R025346be9d504e62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc99f3efe277d4394"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="调用明细" sheetId="2" r:id="Ra2434ea4b94c43f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="汇总" sheetId="3" r:id="Rdbe2a210dd464a6b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2189,17 +2189,26 @@
     <x:col min="6" max="16384" width="8.75" style="1" customWidth="0"/>
     <x:col min="6" max="6" width="10" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="46" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="24" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="24" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="24" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="24" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="24" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="24" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="16" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="16" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="34" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="18" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="18" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="18" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="18" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="18" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="18" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="18" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="18" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="18" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="18" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="18" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="18" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="18" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="16" hidden="0" customWidth="1"/>
+    <x:col min="26" max="26" width="16" hidden="0" customWidth="1"/>
+    <x:col min="27" max="27" width="34" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
@@ -2225,36 +2234,63 @@
         <x:v>转换后问题（Workflow inputText/query）</x:v>
       </x:c>
       <x:c r="H1" s="19" t="str">
-        <x:v>AICO Tool Call - Skill</x:v>
+        <x:v>AICO Skill 第1次(ms)</x:v>
       </x:c>
       <x:c r="I1" s="19" t="str">
-        <x:v>AICO Tool Call - Workflow</x:v>
+        <x:v>AICO Workflow 第1次(ms)</x:v>
       </x:c>
       <x:c r="J1" s="19" t="str">
-        <x:v>Recipe - DeepSeek</x:v>
+        <x:v>Recipe DeepSeek 第1次(ms)</x:v>
       </x:c>
       <x:c r="K1" s="19" t="str">
-        <x:v>Recipe - Qwen执行（最后一次之前）</x:v>
+        <x:v>Recipe DeepSeek 第2次(ms)</x:v>
       </x:c>
       <x:c r="L1" s="19" t="str">
-        <x:v>Recipe - Qwen总结（最后一次）</x:v>
+        <x:v>Recipe DeepSeek 第3次(ms)</x:v>
       </x:c>
       <x:c r="M1" s="19" t="str">
-        <x:v>AICO总结</x:v>
+        <x:v>Recipe DeepSeek 第4次(ms)</x:v>
       </x:c>
       <x:c r="N1" s="19" t="str">
-        <x:v>问题推荐</x:v>
+        <x:v>Recipe DeepSeek 第5次(ms)</x:v>
       </x:c>
       <x:c r="O1" s="19" t="str">
-        <x:v>AICO其他工具</x:v>
+        <x:v>Recipe DeepSeek 第6次(ms)</x:v>
       </x:c>
       <x:c r="P1" s="19" t="str">
+        <x:v>Recipe Qwen执行 第1次(ms)</x:v>
+      </x:c>
+      <x:c r="Q1" s="19" t="str">
+        <x:v>Recipe Qwen执行 第2次(ms)</x:v>
+      </x:c>
+      <x:c r="R1" s="19" t="str">
+        <x:v>Recipe Qwen总结 第1次(ms)</x:v>
+      </x:c>
+      <x:c r="S1" s="19" t="str">
+        <x:v>AICO总结 第1次(ms)</x:v>
+      </x:c>
+      <x:c r="T1" s="19" t="str">
+        <x:v>问题推荐 第1次(ms)</x:v>
+      </x:c>
+      <x:c r="U1" s="19" t="str">
+        <x:v>AICO其他工具 第1次(ms)</x:v>
+      </x:c>
+      <x:c r="V1" s="19" t="str">
+        <x:v>AICO其他工具 第2次(ms)</x:v>
+      </x:c>
+      <x:c r="W1" s="19" t="str">
+        <x:v>AICO其他工具 第3次(ms)</x:v>
+      </x:c>
+      <x:c r="X1" s="19" t="str">
+        <x:v>AICO错误/失败 第1次(ms)</x:v>
+      </x:c>
+      <x:c r="Y1" s="19" t="str">
         <x:v>模型调用总时延(ms)</x:v>
       </x:c>
-      <x:c r="Q1" s="19" t="str">
+      <x:c r="Z1" s="19" t="str">
         <x:v>模型调用次数</x:v>
       </x:c>
-      <x:c r="R1" s="20" t="str">
+      <x:c r="AA1" s="20" t="str">
         <x:v>流程完整性</x:v>
       </x:c>
     </x:row>
@@ -2280,39 +2316,46 @@
       <x:c r="G2" s="23" t="str">
         <x:v>查询深圳大梅沙D-HRH-2小区的经度、纬度和方位角</x:v>
       </x:c>
-      <x:c r="H2" s="23" t="str">
-        <x:v>2558.2 ms</x:v>
-      </x:c>
-      <x:c r="I2" s="23" t="str">
-        <x:v>2664.2 ms</x:v>
-      </x:c>
-      <x:c r="J2" s="23" t="str">
-        <x:v>1438.7 ms</x:v>
-      </x:c>
-      <x:c r="K2" s="23" t="str">
-        <x:v>1246.8 ms</x:v>
-      </x:c>
-      <x:c r="L2" s="23" t="str">
-        <x:v>1554.4 ms</x:v>
-      </x:c>
-      <x:c r="M2" s="23" t="str">
-        <x:v>2325.2 ms</x:v>
-      </x:c>
-      <x:c r="N2" s="23" t="str">
-        <x:v>3228.9 ms</x:v>
-      </x:c>
-      <x:c r="O2" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H2" s="27" t="n">
+        <x:v>2558.21</x:v>
+      </x:c>
+      <x:c r="I2" s="27" t="n">
+        <x:v>2664.238</x:v>
+      </x:c>
+      <x:c r="J2" s="27" t="n">
+        <x:v>1438.719</x:v>
+      </x:c>
+      <x:c r="K2" s="27"/>
+      <x:c r="L2" s="27"/>
+      <x:c r="M2" s="27"/>
+      <x:c r="N2" s="27"/>
+      <x:c r="O2" s="27"/>
       <x:c r="P2" s="27" t="n">
+        <x:v>1246.79</x:v>
+      </x:c>
+      <x:c r="Q2" s="27"/>
+      <x:c r="R2" s="27" t="n">
+        <x:v>1554.401</x:v>
+      </x:c>
+      <x:c r="S2" s="27" t="n">
+        <x:v>2325.197</x:v>
+      </x:c>
+      <x:c r="T2" s="27" t="n">
+        <x:v>3228.881</x:v>
+      </x:c>
+      <x:c r="U2" s="27"/>
+      <x:c r="V2" s="27"/>
+      <x:c r="W2" s="27"/>
+      <x:c r="X2" s="27"/>
+      <x:c r="Y2" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F2,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>15016.436</x:v>
       </x:c>
-      <x:c r="Q2" s="27" t="n">
+      <x:c r="Z2" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F2)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R2" s="23" t="str">
+      <x:c r="AA2" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2338,39 +2381,46 @@
       <x:c r="G3" s="23" t="str">
         <x:v>查询CBN-深圳天麓八区U-H5H站点下所有小区的天线高度和机械下倾角</x:v>
       </x:c>
-      <x:c r="H3" s="23" t="str">
-        <x:v>3182.4 ms</x:v>
-      </x:c>
-      <x:c r="I3" s="23" t="str">
-        <x:v>2616.2 ms</x:v>
-      </x:c>
-      <x:c r="J3" s="23" t="str">
-        <x:v>1560.1 ms</x:v>
-      </x:c>
-      <x:c r="K3" s="23" t="str">
-        <x:v>1255.0 ms</x:v>
-      </x:c>
-      <x:c r="L3" s="23" t="str">
-        <x:v>1476.3 ms</x:v>
-      </x:c>
-      <x:c r="M3" s="23" t="str">
-        <x:v>2215.8 ms</x:v>
-      </x:c>
-      <x:c r="N3" s="23" t="str">
-        <x:v>3098.8 ms</x:v>
-      </x:c>
-      <x:c r="O3" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H3" s="27" t="n">
+        <x:v>3182.448</x:v>
+      </x:c>
+      <x:c r="I3" s="27" t="n">
+        <x:v>2616.175</x:v>
+      </x:c>
+      <x:c r="J3" s="27" t="n">
+        <x:v>1560.145</x:v>
+      </x:c>
+      <x:c r="K3" s="27"/>
+      <x:c r="L3" s="27"/>
+      <x:c r="M3" s="27"/>
+      <x:c r="N3" s="27"/>
+      <x:c r="O3" s="27"/>
       <x:c r="P3" s="27" t="n">
+        <x:v>1255.006</x:v>
+      </x:c>
+      <x:c r="Q3" s="27"/>
+      <x:c r="R3" s="27" t="n">
+        <x:v>1476.259</x:v>
+      </x:c>
+      <x:c r="S3" s="27" t="n">
+        <x:v>2215.754</x:v>
+      </x:c>
+      <x:c r="T3" s="27" t="n">
+        <x:v>3098.838</x:v>
+      </x:c>
+      <x:c r="U3" s="27"/>
+      <x:c r="V3" s="27"/>
+      <x:c r="W3" s="27"/>
+      <x:c r="X3" s="27"/>
+      <x:c r="Y3" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F3,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>15404.625</x:v>
       </x:c>
-      <x:c r="Q3" s="27" t="n">
+      <x:c r="Z3" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F3)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R3" s="23" t="str">
+      <x:c r="AA3" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2396,39 +2446,46 @@
       <x:c r="G4" s="23" t="str">
         <x:v>查询CBN-福州仓山-火车南站西广场南侧高架桥旁C-HRHH-512小区的小区标识和基站标识。</x:v>
       </x:c>
-      <x:c r="H4" s="23" t="str">
-        <x:v>2969.0 ms</x:v>
-      </x:c>
-      <x:c r="I4" s="23" t="str">
-        <x:v>3100.5 ms</x:v>
-      </x:c>
-      <x:c r="J4" s="23" t="str">
-        <x:v>1958.7 ms</x:v>
-      </x:c>
-      <x:c r="K4" s="23" t="str">
-        <x:v>1334.0 ms</x:v>
-      </x:c>
-      <x:c r="L4" s="23" t="str">
-        <x:v>1604.3 ms</x:v>
-      </x:c>
-      <x:c r="M4" s="23" t="str">
-        <x:v>2102.9 ms</x:v>
-      </x:c>
-      <x:c r="N4" s="23" t="str">
-        <x:v>3096.5 ms</x:v>
-      </x:c>
-      <x:c r="O4" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H4" s="27" t="n">
+        <x:v>2969.035</x:v>
+      </x:c>
+      <x:c r="I4" s="27" t="n">
+        <x:v>3100.513</x:v>
+      </x:c>
+      <x:c r="J4" s="27" t="n">
+        <x:v>1958.677</x:v>
+      </x:c>
+      <x:c r="K4" s="27"/>
+      <x:c r="L4" s="27"/>
+      <x:c r="M4" s="27"/>
+      <x:c r="N4" s="27"/>
+      <x:c r="O4" s="27"/>
       <x:c r="P4" s="27" t="n">
+        <x:v>1333.99</x:v>
+      </x:c>
+      <x:c r="Q4" s="27"/>
+      <x:c r="R4" s="27" t="n">
+        <x:v>1604.293</x:v>
+      </x:c>
+      <x:c r="S4" s="27" t="n">
+        <x:v>2102.938</x:v>
+      </x:c>
+      <x:c r="T4" s="27" t="n">
+        <x:v>3096.492</x:v>
+      </x:c>
+      <x:c r="U4" s="27"/>
+      <x:c r="V4" s="27"/>
+      <x:c r="W4" s="27"/>
+      <x:c r="X4" s="27"/>
+      <x:c r="Y4" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F4,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>16165.938</x:v>
       </x:c>
-      <x:c r="Q4" s="27" t="n">
+      <x:c r="Z4" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F4)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R4" s="23" t="str">
+      <x:c r="AA4" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2454,39 +2511,46 @@
       <x:c r="G5" s="23" t="str">
         <x:v>查询深圳梅沙湾二D-HRH-3小区的方向角是多少</x:v>
       </x:c>
-      <x:c r="H5" s="23" t="str">
-        <x:v>2510.2 ms</x:v>
-      </x:c>
-      <x:c r="I5" s="23" t="str">
-        <x:v>2476.4 ms</x:v>
-      </x:c>
-      <x:c r="J5" s="23" t="str">
-        <x:v>1423.2 ms</x:v>
-      </x:c>
-      <x:c r="K5" s="23" t="str">
-        <x:v>1175.7 ms</x:v>
-      </x:c>
-      <x:c r="L5" s="23" t="str">
-        <x:v>1252.7 ms</x:v>
-      </x:c>
-      <x:c r="M5" s="23" t="str">
-        <x:v>1913.8 ms</x:v>
-      </x:c>
-      <x:c r="N5" s="23" t="str">
-        <x:v>2920.2 ms</x:v>
-      </x:c>
-      <x:c r="O5" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H5" s="27" t="n">
+        <x:v>2510.237</x:v>
+      </x:c>
+      <x:c r="I5" s="27" t="n">
+        <x:v>2476.434</x:v>
+      </x:c>
+      <x:c r="J5" s="27" t="n">
+        <x:v>1423.216</x:v>
+      </x:c>
+      <x:c r="K5" s="27"/>
+      <x:c r="L5" s="27"/>
+      <x:c r="M5" s="27"/>
+      <x:c r="N5" s="27"/>
+      <x:c r="O5" s="27"/>
       <x:c r="P5" s="27" t="n">
+        <x:v>1175.743</x:v>
+      </x:c>
+      <x:c r="Q5" s="27"/>
+      <x:c r="R5" s="27" t="n">
+        <x:v>1252.695</x:v>
+      </x:c>
+      <x:c r="S5" s="27" t="n">
+        <x:v>1913.771</x:v>
+      </x:c>
+      <x:c r="T5" s="27" t="n">
+        <x:v>2920.227</x:v>
+      </x:c>
+      <x:c r="U5" s="27"/>
+      <x:c r="V5" s="27"/>
+      <x:c r="W5" s="27"/>
+      <x:c r="X5" s="27"/>
+      <x:c r="Y5" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F5,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>13672.323</x:v>
       </x:c>
-      <x:c r="Q5" s="27" t="n">
+      <x:c r="Z5" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F5)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R5" s="23" t="str">
+      <x:c r="AA5" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2512,39 +2576,46 @@
       <x:c r="G6" s="23" t="str">
         <x:v>查询CBN-福州晋安-高铁鼓山1号隧道洞室1C-HRRH站点下所有小区的经度和纬度。</x:v>
       </x:c>
-      <x:c r="H6" s="23" t="str">
-        <x:v>2971.0 ms</x:v>
-      </x:c>
-      <x:c r="I6" s="23" t="str">
-        <x:v>2812.1 ms</x:v>
-      </x:c>
-      <x:c r="J6" s="23" t="str">
-        <x:v>1710.7 ms</x:v>
-      </x:c>
-      <x:c r="K6" s="23" t="str">
-        <x:v>1278.2 ms</x:v>
-      </x:c>
-      <x:c r="L6" s="23" t="str">
-        <x:v>2757.2 ms</x:v>
-      </x:c>
-      <x:c r="M6" s="23" t="str">
-        <x:v>3462.6 ms</x:v>
-      </x:c>
-      <x:c r="N6" s="23" t="str">
-        <x:v>2816.2 ms</x:v>
-      </x:c>
-      <x:c r="O6" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H6" s="27" t="n">
+        <x:v>2971.033</x:v>
+      </x:c>
+      <x:c r="I6" s="27" t="n">
+        <x:v>2812.062</x:v>
+      </x:c>
+      <x:c r="J6" s="27" t="n">
+        <x:v>1710.739</x:v>
+      </x:c>
+      <x:c r="K6" s="27"/>
+      <x:c r="L6" s="27"/>
+      <x:c r="M6" s="27"/>
+      <x:c r="N6" s="27"/>
+      <x:c r="O6" s="27"/>
       <x:c r="P6" s="27" t="n">
+        <x:v>1278.239</x:v>
+      </x:c>
+      <x:c r="Q6" s="27"/>
+      <x:c r="R6" s="27" t="n">
+        <x:v>2757.217</x:v>
+      </x:c>
+      <x:c r="S6" s="27" t="n">
+        <x:v>3462.602</x:v>
+      </x:c>
+      <x:c r="T6" s="27" t="n">
+        <x:v>2816.211</x:v>
+      </x:c>
+      <x:c r="U6" s="27"/>
+      <x:c r="V6" s="27"/>
+      <x:c r="W6" s="27"/>
+      <x:c r="X6" s="27"/>
+      <x:c r="Y6" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F6,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>17808.103</x:v>
       </x:c>
-      <x:c r="Q6" s="27" t="n">
+      <x:c r="Z6" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F6)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R6" s="23" t="str">
+      <x:c r="AA6" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2570,39 +2641,46 @@
       <x:c r="G7" s="23" t="str">
         <x:v>查询CBN-福州晋安-福厦高铁苔井山隧道入口（左侧）C-HRRH-513和CBN-福州仓山-福厦高铁鸡笼山隧道C-HRRH-513这两个小区的方位角、电子下倾角和机械下倾角。</x:v>
       </x:c>
-      <x:c r="H7" s="23" t="str">
-        <x:v>3170.3 ms</x:v>
-      </x:c>
-      <x:c r="I7" s="23" t="str">
-        <x:v>3103.7 ms</x:v>
-      </x:c>
-      <x:c r="J7" s="23" t="str">
-        <x:v>2300.6 ms</x:v>
-      </x:c>
-      <x:c r="K7" s="23" t="str">
-        <x:v>1808.7 ms</x:v>
-      </x:c>
-      <x:c r="L7" s="23" t="str">
-        <x:v>1885.8 ms</x:v>
-      </x:c>
-      <x:c r="M7" s="23" t="str">
-        <x:v>2793.5 ms</x:v>
-      </x:c>
-      <x:c r="N7" s="23" t="str">
-        <x:v>3707.1 ms</x:v>
-      </x:c>
-      <x:c r="O7" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H7" s="27" t="n">
+        <x:v>3170.303</x:v>
+      </x:c>
+      <x:c r="I7" s="27" t="n">
+        <x:v>3103.728</x:v>
+      </x:c>
+      <x:c r="J7" s="27" t="n">
+        <x:v>2300.612</x:v>
+      </x:c>
+      <x:c r="K7" s="27"/>
+      <x:c r="L7" s="27"/>
+      <x:c r="M7" s="27"/>
+      <x:c r="N7" s="27"/>
+      <x:c r="O7" s="27"/>
       <x:c r="P7" s="27" t="n">
+        <x:v>1808.691</x:v>
+      </x:c>
+      <x:c r="Q7" s="27"/>
+      <x:c r="R7" s="27" t="n">
+        <x:v>1885.766</x:v>
+      </x:c>
+      <x:c r="S7" s="27" t="n">
+        <x:v>2793.53</x:v>
+      </x:c>
+      <x:c r="T7" s="27" t="n">
+        <x:v>3707.069</x:v>
+      </x:c>
+      <x:c r="U7" s="27"/>
+      <x:c r="V7" s="27"/>
+      <x:c r="W7" s="27"/>
+      <x:c r="X7" s="27"/>
+      <x:c r="Y7" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F7,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18769.699</x:v>
       </x:c>
-      <x:c r="Q7" s="27" t="n">
+      <x:c r="Z7" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F7)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R7" s="23" t="str">
+      <x:c r="AA7" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2628,39 +2706,48 @@
       <x:c r="G8" s="23" t="str">
         <x:v>查询深圳东华风车D-HRH和CBN-深圳上威梅沙二U-H5H这两个站点下小区的基站标识、纬度和设备厂商</x:v>
       </x:c>
-      <x:c r="H8" s="23" t="str">
-        <x:v>3273.0 ms</x:v>
-      </x:c>
-      <x:c r="I8" s="23" t="str">
-        <x:v>2795.2 ms</x:v>
-      </x:c>
-      <x:c r="J8" s="23" t="str">
-        <x:v>1827.3 ms</x:v>
-      </x:c>
-      <x:c r="K8" s="23" t="str">
-        <x:v>第1次 1310.6 ms；第2次 1486.0 ms</x:v>
-      </x:c>
-      <x:c r="L8" s="23" t="str">
-        <x:v>2814.5 ms</x:v>
-      </x:c>
-      <x:c r="M8" s="23" t="str">
-        <x:v>3585.7 ms</x:v>
-      </x:c>
-      <x:c r="N8" s="23" t="str">
-        <x:v>2983.4 ms</x:v>
-      </x:c>
-      <x:c r="O8" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H8" s="27" t="n">
+        <x:v>3273.024</x:v>
+      </x:c>
+      <x:c r="I8" s="27" t="n">
+        <x:v>2795.167</x:v>
+      </x:c>
+      <x:c r="J8" s="27" t="n">
+        <x:v>1827.254</x:v>
+      </x:c>
+      <x:c r="K8" s="27"/>
+      <x:c r="L8" s="27"/>
+      <x:c r="M8" s="27"/>
+      <x:c r="N8" s="27"/>
+      <x:c r="O8" s="27"/>
       <x:c r="P8" s="27" t="n">
+        <x:v>1310.557</x:v>
+      </x:c>
+      <x:c r="Q8" s="27" t="n">
+        <x:v>1485.998</x:v>
+      </x:c>
+      <x:c r="R8" s="27" t="n">
+        <x:v>2814.549</x:v>
+      </x:c>
+      <x:c r="S8" s="27" t="n">
+        <x:v>3585.743</x:v>
+      </x:c>
+      <x:c r="T8" s="27" t="n">
+        <x:v>2983.439</x:v>
+      </x:c>
+      <x:c r="U8" s="27"/>
+      <x:c r="V8" s="27"/>
+      <x:c r="W8" s="27"/>
+      <x:c r="X8" s="27"/>
+      <x:c r="Y8" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F8,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>20075.730999999996</x:v>
       </x:c>
-      <x:c r="Q8" s="27" t="n">
+      <x:c r="Z8" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F8)</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="R8" s="23" t="str">
+      <x:c r="AA8" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2686,39 +2773,46 @@
       <x:c r="G9" s="23" t="str">
         <x:v>查询小区 CBN-深圳梅沙湾U-H5H-0712、CBN-深圳梅沙湾U-H5H-0711 和 CBN-深圳东海岸三[CBN-深圳天麓八区U-H5H]U-H5H-0711 这三个小区的移动国家码、方向角和天线高度。</x:v>
       </x:c>
-      <x:c r="H9" s="23" t="str">
-        <x:v>3436.5 ms</x:v>
-      </x:c>
-      <x:c r="I9" s="23" t="str">
-        <x:v>3048.2 ms</x:v>
-      </x:c>
-      <x:c r="J9" s="23" t="str">
-        <x:v>2524.3 ms</x:v>
-      </x:c>
-      <x:c r="K9" s="23" t="str">
-        <x:v>1899.2 ms</x:v>
-      </x:c>
-      <x:c r="L9" s="23" t="str">
-        <x:v>2490.7 ms</x:v>
-      </x:c>
-      <x:c r="M9" s="23" t="str">
-        <x:v>4276.8 ms</x:v>
-      </x:c>
-      <x:c r="N9" s="23" t="str">
-        <x:v>2772.4 ms</x:v>
-      </x:c>
-      <x:c r="O9" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H9" s="27" t="n">
+        <x:v>3436.476</x:v>
+      </x:c>
+      <x:c r="I9" s="27" t="n">
+        <x:v>3048.185</x:v>
+      </x:c>
+      <x:c r="J9" s="27" t="n">
+        <x:v>2524.313</x:v>
+      </x:c>
+      <x:c r="K9" s="27"/>
+      <x:c r="L9" s="27"/>
+      <x:c r="M9" s="27"/>
+      <x:c r="N9" s="27"/>
+      <x:c r="O9" s="27"/>
       <x:c r="P9" s="27" t="n">
+        <x:v>1899.158</x:v>
+      </x:c>
+      <x:c r="Q9" s="27"/>
+      <x:c r="R9" s="27" t="n">
+        <x:v>2490.734</x:v>
+      </x:c>
+      <x:c r="S9" s="27" t="n">
+        <x:v>4276.82</x:v>
+      </x:c>
+      <x:c r="T9" s="27" t="n">
+        <x:v>2772.373</x:v>
+      </x:c>
+      <x:c r="U9" s="27"/>
+      <x:c r="V9" s="27"/>
+      <x:c r="W9" s="27"/>
+      <x:c r="X9" s="27"/>
+      <x:c r="Y9" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F9,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>20448.059</x:v>
       </x:c>
-      <x:c r="Q9" s="27" t="n">
+      <x:c r="Z9" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F9)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R9" s="23" t="str">
+      <x:c r="AA9" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2744,39 +2838,46 @@
       <x:c r="G10" s="23" t="str">
         <x:v>查询站点CBN-福州晋安-站东路三环北路交叉西C-HRRH和CBN-福州仓山-高铁鸡笼山隧道入口C-HRRH下所有小区的经度、纬度和方位角</x:v>
       </x:c>
-      <x:c r="H10" s="23" t="str">
-        <x:v>3160.8 ms</x:v>
-      </x:c>
-      <x:c r="I10" s="23" t="str">
-        <x:v>2880.1 ms</x:v>
-      </x:c>
-      <x:c r="J10" s="23" t="str">
-        <x:v>2178.7 ms</x:v>
-      </x:c>
-      <x:c r="K10" s="23" t="str">
-        <x:v>1464.2 ms</x:v>
-      </x:c>
-      <x:c r="L10" s="23" t="str">
-        <x:v>3410.7 ms</x:v>
-      </x:c>
-      <x:c r="M10" s="23" t="str">
-        <x:v>4721.9 ms</x:v>
-      </x:c>
-      <x:c r="N10" s="23" t="str">
-        <x:v>4069.4 ms</x:v>
-      </x:c>
-      <x:c r="O10" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H10" s="27" t="n">
+        <x:v>3160.758</x:v>
+      </x:c>
+      <x:c r="I10" s="27" t="n">
+        <x:v>2880.131</x:v>
+      </x:c>
+      <x:c r="J10" s="27" t="n">
+        <x:v>2178.716</x:v>
+      </x:c>
+      <x:c r="K10" s="27"/>
+      <x:c r="L10" s="27"/>
+      <x:c r="M10" s="27"/>
+      <x:c r="N10" s="27"/>
+      <x:c r="O10" s="27"/>
       <x:c r="P10" s="27" t="n">
+        <x:v>1464.228</x:v>
+      </x:c>
+      <x:c r="Q10" s="27"/>
+      <x:c r="R10" s="27" t="n">
+        <x:v>3410.687</x:v>
+      </x:c>
+      <x:c r="S10" s="27" t="n">
+        <x:v>4721.901</x:v>
+      </x:c>
+      <x:c r="T10" s="27" t="n">
+        <x:v>4069.377</x:v>
+      </x:c>
+      <x:c r="U10" s="27"/>
+      <x:c r="V10" s="27"/>
+      <x:c r="W10" s="27"/>
+      <x:c r="X10" s="27"/>
+      <x:c r="Y10" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F10,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>21885.798</x:v>
       </x:c>
-      <x:c r="Q10" s="27" t="n">
+      <x:c r="Z10" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F10)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R10" s="23" t="str">
+      <x:c r="AA10" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2802,39 +2903,46 @@
       <x:c r="G11" s="23" t="str">
         <x:v>查询小区 CBN-福州晋安-东浦新村4号楼C-HRHH-512、CBN-福州晋安-东浦新村4号楼C-HRHH-514 和 深圳大梅沙D-HRH-3 这三个小区的站点名称、小区标识和电子下倾角。</x:v>
       </x:c>
-      <x:c r="H11" s="23" t="str">
-        <x:v>3984.8 ms</x:v>
-      </x:c>
-      <x:c r="I11" s="23" t="str">
-        <x:v>3159.4 ms</x:v>
-      </x:c>
-      <x:c r="J11" s="23" t="str">
-        <x:v>2357.2 ms</x:v>
-      </x:c>
-      <x:c r="K11" s="23" t="str">
-        <x:v>1883.7 ms</x:v>
-      </x:c>
-      <x:c r="L11" s="23" t="str">
-        <x:v>2287.3 ms</x:v>
-      </x:c>
-      <x:c r="M11" s="23" t="str">
-        <x:v>3589.1 ms</x:v>
-      </x:c>
-      <x:c r="N11" s="23" t="str">
-        <x:v>3472.5 ms</x:v>
-      </x:c>
-      <x:c r="O11" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H11" s="27" t="n">
+        <x:v>3984.808</x:v>
+      </x:c>
+      <x:c r="I11" s="27" t="n">
+        <x:v>3159.428</x:v>
+      </x:c>
+      <x:c r="J11" s="27" t="n">
+        <x:v>2357.211</x:v>
+      </x:c>
+      <x:c r="K11" s="27"/>
+      <x:c r="L11" s="27"/>
+      <x:c r="M11" s="27"/>
+      <x:c r="N11" s="27"/>
+      <x:c r="O11" s="27"/>
       <x:c r="P11" s="27" t="n">
+        <x:v>1883.677</x:v>
+      </x:c>
+      <x:c r="Q11" s="27"/>
+      <x:c r="R11" s="27" t="n">
+        <x:v>2287.266</x:v>
+      </x:c>
+      <x:c r="S11" s="27" t="n">
+        <x:v>3589.051</x:v>
+      </x:c>
+      <x:c r="T11" s="27" t="n">
+        <x:v>3472.471</x:v>
+      </x:c>
+      <x:c r="U11" s="27"/>
+      <x:c r="V11" s="27"/>
+      <x:c r="W11" s="27"/>
+      <x:c r="X11" s="27"/>
+      <x:c r="Y11" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F11,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>20733.912</x:v>
       </x:c>
-      <x:c r="Q11" s="27" t="n">
+      <x:c r="Z11" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F11)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R11" s="23" t="str">
+      <x:c r="AA11" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2860,39 +2968,46 @@
       <x:c r="G12" s="23" t="str">
         <x:v>查询CBN-深圳大梅沙U-H5H站点下5G小区的小区名称、基站标识和方位角</x:v>
       </x:c>
-      <x:c r="H12" s="23" t="str">
-        <x:v>2816.4 ms</x:v>
-      </x:c>
-      <x:c r="I12" s="23" t="str">
-        <x:v>2807.9 ms</x:v>
-      </x:c>
-      <x:c r="J12" s="23" t="str">
-        <x:v>1687.1 ms</x:v>
-      </x:c>
-      <x:c r="K12" s="23" t="str">
-        <x:v>1380.1 ms</x:v>
-      </x:c>
-      <x:c r="L12" s="23" t="str">
-        <x:v>2583.8 ms</x:v>
-      </x:c>
-      <x:c r="M12" s="23" t="str">
-        <x:v>6576.3 ms</x:v>
-      </x:c>
-      <x:c r="N12" s="23" t="str">
-        <x:v>3552.0 ms</x:v>
-      </x:c>
-      <x:c r="O12" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H12" s="27" t="n">
+        <x:v>2816.38</x:v>
+      </x:c>
+      <x:c r="I12" s="27" t="n">
+        <x:v>2807.909</x:v>
+      </x:c>
+      <x:c r="J12" s="27" t="n">
+        <x:v>1687.119</x:v>
+      </x:c>
+      <x:c r="K12" s="27"/>
+      <x:c r="L12" s="27"/>
+      <x:c r="M12" s="27"/>
+      <x:c r="N12" s="27"/>
+      <x:c r="O12" s="27"/>
       <x:c r="P12" s="27" t="n">
+        <x:v>1380.091</x:v>
+      </x:c>
+      <x:c r="Q12" s="27"/>
+      <x:c r="R12" s="27" t="n">
+        <x:v>2583.843</x:v>
+      </x:c>
+      <x:c r="S12" s="27" t="n">
+        <x:v>6576.342</x:v>
+      </x:c>
+      <x:c r="T12" s="27" t="n">
+        <x:v>3551.99</x:v>
+      </x:c>
+      <x:c r="U12" s="27"/>
+      <x:c r="V12" s="27"/>
+      <x:c r="W12" s="27"/>
+      <x:c r="X12" s="27"/>
+      <x:c r="Y12" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F12,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>21403.674</x:v>
       </x:c>
-      <x:c r="Q12" s="27" t="n">
+      <x:c r="Z12" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F12)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R12" s="23" t="str">
+      <x:c r="AA12" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2918,39 +3033,46 @@
       <x:c r="G13" s="23" t="str">
         <x:v>查询深圳大梅沙二[深圳大梅沙二D-HRH]C-HRH-3这个NR小区的机械下倾角、电子下倾角和天线高度工程参数。</x:v>
       </x:c>
-      <x:c r="H13" s="23" t="str">
-        <x:v>3448.3 ms</x:v>
-      </x:c>
-      <x:c r="I13" s="23" t="str">
-        <x:v>3292.7 ms</x:v>
-      </x:c>
-      <x:c r="J13" s="23" t="str">
-        <x:v>2619.6 ms</x:v>
-      </x:c>
-      <x:c r="K13" s="23" t="str">
-        <x:v>1725.0 ms</x:v>
-      </x:c>
-      <x:c r="L13" s="23" t="str">
-        <x:v>1555.1 ms</x:v>
-      </x:c>
-      <x:c r="M13" s="23" t="str">
-        <x:v>2212.8 ms</x:v>
-      </x:c>
-      <x:c r="N13" s="23" t="str">
-        <x:v>3902.5 ms</x:v>
-      </x:c>
-      <x:c r="O13" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H13" s="27" t="n">
+        <x:v>3448.282</x:v>
+      </x:c>
+      <x:c r="I13" s="27" t="n">
+        <x:v>3292.689</x:v>
+      </x:c>
+      <x:c r="J13" s="27" t="n">
+        <x:v>2619.62</x:v>
+      </x:c>
+      <x:c r="K13" s="27"/>
+      <x:c r="L13" s="27"/>
+      <x:c r="M13" s="27"/>
+      <x:c r="N13" s="27"/>
+      <x:c r="O13" s="27"/>
       <x:c r="P13" s="27" t="n">
+        <x:v>1724.985</x:v>
+      </x:c>
+      <x:c r="Q13" s="27"/>
+      <x:c r="R13" s="27" t="n">
+        <x:v>1555.126</x:v>
+      </x:c>
+      <x:c r="S13" s="27" t="n">
+        <x:v>2212.759</x:v>
+      </x:c>
+      <x:c r="T13" s="27" t="n">
+        <x:v>3902.505</x:v>
+      </x:c>
+      <x:c r="U13" s="27"/>
+      <x:c r="V13" s="27"/>
+      <x:c r="W13" s="27"/>
+      <x:c r="X13" s="27"/>
+      <x:c r="Y13" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F13,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18755.966</x:v>
       </x:c>
-      <x:c r="Q13" s="27" t="n">
+      <x:c r="Z13" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F13)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R13" s="23" t="str">
+      <x:c r="AA13" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -2976,39 +3098,48 @@
       <x:c r="G14" s="23" t="str">
         <x:v>查询CBN-福州晋安-站东路三环北路交叉西C-HRRH和深圳东海岸三D-HRH这两个站点下5G小区的纬度、经度和设备厂商。</x:v>
       </x:c>
-      <x:c r="H14" s="23" t="str">
-        <x:v>3381.9 ms</x:v>
-      </x:c>
-      <x:c r="I14" s="23" t="str">
-        <x:v>6551.5 ms</x:v>
-      </x:c>
-      <x:c r="J14" s="23" t="str">
-        <x:v>3005.0 ms</x:v>
-      </x:c>
-      <x:c r="K14" s="23" t="str">
-        <x:v>第1次 1442.8 ms；第2次 1870.4 ms</x:v>
-      </x:c>
-      <x:c r="L14" s="23" t="str">
-        <x:v>3328.3 ms</x:v>
-      </x:c>
-      <x:c r="M14" s="23" t="str">
-        <x:v>3888.9 ms</x:v>
-      </x:c>
-      <x:c r="N14" s="23" t="str">
-        <x:v>3610.2 ms</x:v>
-      </x:c>
-      <x:c r="O14" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H14" s="27" t="n">
+        <x:v>3381.877</x:v>
+      </x:c>
+      <x:c r="I14" s="27" t="n">
+        <x:v>6551.514</x:v>
+      </x:c>
+      <x:c r="J14" s="27" t="n">
+        <x:v>3004.979</x:v>
+      </x:c>
+      <x:c r="K14" s="27"/>
+      <x:c r="L14" s="27"/>
+      <x:c r="M14" s="27"/>
+      <x:c r="N14" s="27"/>
+      <x:c r="O14" s="27"/>
       <x:c r="P14" s="27" t="n">
+        <x:v>1442.822</x:v>
+      </x:c>
+      <x:c r="Q14" s="27" t="n">
+        <x:v>1870.355</x:v>
+      </x:c>
+      <x:c r="R14" s="27" t="n">
+        <x:v>3328.325</x:v>
+      </x:c>
+      <x:c r="S14" s="27" t="n">
+        <x:v>3888.925</x:v>
+      </x:c>
+      <x:c r="T14" s="27" t="n">
+        <x:v>3610.203</x:v>
+      </x:c>
+      <x:c r="U14" s="27"/>
+      <x:c r="V14" s="27"/>
+      <x:c r="W14" s="27"/>
+      <x:c r="X14" s="27"/>
+      <x:c r="Y14" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F14,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>27079</x:v>
       </x:c>
-      <x:c r="Q14" s="27" t="n">
+      <x:c r="Z14" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F14)</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="R14" s="23" t="str">
+      <x:c r="AA14" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3034,39 +3165,46 @@
       <x:c r="G15" s="23" t="str">
         <x:v>查询CBN-福州仓山-福州火车南站C-HRHH-521和CBN-福州晋安-东浦新村4号楼C-HRHH-513这两个NR小区的方向角、移动国家码和站点名称。</x:v>
       </x:c>
-      <x:c r="H15" s="23" t="str">
-        <x:v>3334.0 ms</x:v>
-      </x:c>
-      <x:c r="I15" s="23" t="str">
-        <x:v>2890.7 ms</x:v>
-      </x:c>
-      <x:c r="J15" s="23" t="str">
-        <x:v>2154.0 ms</x:v>
-      </x:c>
-      <x:c r="K15" s="23" t="str">
-        <x:v>1826.9 ms</x:v>
-      </x:c>
-      <x:c r="L15" s="23" t="str">
-        <x:v>1945.2 ms</x:v>
-      </x:c>
-      <x:c r="M15" s="23" t="str">
-        <x:v>2969.3 ms</x:v>
-      </x:c>
-      <x:c r="N15" s="23" t="str">
-        <x:v>2968.1 ms</x:v>
-      </x:c>
-      <x:c r="O15" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H15" s="27" t="n">
+        <x:v>3334.016</x:v>
+      </x:c>
+      <x:c r="I15" s="27" t="n">
+        <x:v>2890.723</x:v>
+      </x:c>
+      <x:c r="J15" s="27" t="n">
+        <x:v>2154.014</x:v>
+      </x:c>
+      <x:c r="K15" s="27"/>
+      <x:c r="L15" s="27"/>
+      <x:c r="M15" s="27"/>
+      <x:c r="N15" s="27"/>
+      <x:c r="O15" s="27"/>
       <x:c r="P15" s="27" t="n">
+        <x:v>1826.875</x:v>
+      </x:c>
+      <x:c r="Q15" s="27"/>
+      <x:c r="R15" s="27" t="n">
+        <x:v>1945.152</x:v>
+      </x:c>
+      <x:c r="S15" s="27" t="n">
+        <x:v>2969.313</x:v>
+      </x:c>
+      <x:c r="T15" s="27" t="n">
+        <x:v>2968.093</x:v>
+      </x:c>
+      <x:c r="U15" s="27"/>
+      <x:c r="V15" s="27"/>
+      <x:c r="W15" s="27"/>
+      <x:c r="X15" s="27"/>
+      <x:c r="Y15" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F15,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18088.186</x:v>
       </x:c>
-      <x:c r="Q15" s="27" t="n">
+      <x:c r="Z15" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F15)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R15" s="23" t="str">
+      <x:c r="AA15" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3092,39 +3230,46 @@
       <x:c r="G16" s="23" t="str">
         <x:v>查询CBN-深圳梅沙湾二U-H5H站点下5G小区的CGI、小区标识和机械下倾角</x:v>
       </x:c>
-      <x:c r="H16" s="23" t="str">
-        <x:v>3218.9 ms</x:v>
-      </x:c>
-      <x:c r="I16" s="23" t="str">
-        <x:v>2750.1 ms</x:v>
-      </x:c>
-      <x:c r="J16" s="23" t="str">
-        <x:v>1828.8 ms</x:v>
-      </x:c>
-      <x:c r="K16" s="23" t="str">
-        <x:v>1372.4 ms</x:v>
-      </x:c>
-      <x:c r="L16" s="23" t="str">
-        <x:v>2919.6 ms</x:v>
-      </x:c>
-      <x:c r="M16" s="23" t="str">
-        <x:v>3235.7 ms</x:v>
-      </x:c>
-      <x:c r="N16" s="23" t="str">
-        <x:v>3155.3 ms</x:v>
-      </x:c>
-      <x:c r="O16" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H16" s="27" t="n">
+        <x:v>3218.931</x:v>
+      </x:c>
+      <x:c r="I16" s="27" t="n">
+        <x:v>2750.143</x:v>
+      </x:c>
+      <x:c r="J16" s="27" t="n">
+        <x:v>1828.755</x:v>
+      </x:c>
+      <x:c r="K16" s="27"/>
+      <x:c r="L16" s="27"/>
+      <x:c r="M16" s="27"/>
+      <x:c r="N16" s="27"/>
+      <x:c r="O16" s="27"/>
       <x:c r="P16" s="27" t="n">
+        <x:v>1372.403</x:v>
+      </x:c>
+      <x:c r="Q16" s="27"/>
+      <x:c r="R16" s="27" t="n">
+        <x:v>2919.586</x:v>
+      </x:c>
+      <x:c r="S16" s="27" t="n">
+        <x:v>3235.689</x:v>
+      </x:c>
+      <x:c r="T16" s="27" t="n">
+        <x:v>3155.287</x:v>
+      </x:c>
+      <x:c r="U16" s="27"/>
+      <x:c r="V16" s="27"/>
+      <x:c r="W16" s="27"/>
+      <x:c r="X16" s="27"/>
+      <x:c r="Y16" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F16,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18480.793999999998</x:v>
       </x:c>
-      <x:c r="Q16" s="27" t="n">
+      <x:c r="Z16" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F16)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R16" s="23" t="str">
+      <x:c r="AA16" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3150,39 +3295,46 @@
       <x:c r="G17" s="23" t="str">
         <x:v>查询CBN-深圳梅沙湾U-H5H站点下天线高度大于30米的小区，返回小区名称、天线高度和方位角。</x:v>
       </x:c>
-      <x:c r="H17" s="23" t="str">
-        <x:v>3144.1 ms</x:v>
-      </x:c>
-      <x:c r="I17" s="23" t="str">
-        <x:v>2910.8 ms</x:v>
-      </x:c>
-      <x:c r="J17" s="23" t="str">
-        <x:v>1685.4 ms</x:v>
-      </x:c>
-      <x:c r="K17" s="23" t="str">
-        <x:v>1250.0 ms</x:v>
-      </x:c>
-      <x:c r="L17" s="23" t="str">
-        <x:v>1824.4 ms</x:v>
-      </x:c>
-      <x:c r="M17" s="23" t="str">
-        <x:v>2415.5 ms</x:v>
-      </x:c>
-      <x:c r="N17" s="23" t="str">
-        <x:v>3441.5 ms</x:v>
-      </x:c>
-      <x:c r="O17" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H17" s="27" t="n">
+        <x:v>3144.076</x:v>
+      </x:c>
+      <x:c r="I17" s="27" t="n">
+        <x:v>2910.788</x:v>
+      </x:c>
+      <x:c r="J17" s="27" t="n">
+        <x:v>1685.364</x:v>
+      </x:c>
+      <x:c r="K17" s="27"/>
+      <x:c r="L17" s="27"/>
+      <x:c r="M17" s="27"/>
+      <x:c r="N17" s="27"/>
+      <x:c r="O17" s="27"/>
       <x:c r="P17" s="27" t="n">
+        <x:v>1250.004</x:v>
+      </x:c>
+      <x:c r="Q17" s="27"/>
+      <x:c r="R17" s="27" t="n">
+        <x:v>1824.366</x:v>
+      </x:c>
+      <x:c r="S17" s="27" t="n">
+        <x:v>2415.516</x:v>
+      </x:c>
+      <x:c r="T17" s="27" t="n">
+        <x:v>3441.545</x:v>
+      </x:c>
+      <x:c r="U17" s="27"/>
+      <x:c r="V17" s="27"/>
+      <x:c r="W17" s="27"/>
+      <x:c r="X17" s="27"/>
+      <x:c r="Y17" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F17,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>16671.659</x:v>
       </x:c>
-      <x:c r="Q17" s="27" t="n">
+      <x:c r="Z17" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F17)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R17" s="23" t="str">
+      <x:c r="AA17" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3208,39 +3360,46 @@
       <x:c r="G18" s="23" t="str">
         <x:v>查询深圳奥特莱斯D-HRW-1和深圳奥特莱斯D-HRH-2这两个5G小区的机械下倾角、电子下倾角，筛选机械下倾角在3到9之间的小区，返回小区名称、机械下倾角和电子下倾角。</x:v>
       </x:c>
-      <x:c r="H18" s="23" t="str">
-        <x:v>3252.3 ms</x:v>
-      </x:c>
-      <x:c r="I18" s="23" t="str">
-        <x:v>3092.9 ms</x:v>
-      </x:c>
-      <x:c r="J18" s="23" t="str">
-        <x:v>2285.0 ms</x:v>
-      </x:c>
-      <x:c r="K18" s="23" t="str">
-        <x:v>1685.4 ms</x:v>
-      </x:c>
-      <x:c r="L18" s="23" t="str">
-        <x:v>1959.5 ms</x:v>
-      </x:c>
-      <x:c r="M18" s="23" t="str">
-        <x:v>3157.0 ms</x:v>
-      </x:c>
-      <x:c r="N18" s="23" t="str">
-        <x:v>2886.5 ms</x:v>
-      </x:c>
-      <x:c r="O18" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H18" s="27" t="n">
+        <x:v>3252.286</x:v>
+      </x:c>
+      <x:c r="I18" s="27" t="n">
+        <x:v>3092.91</x:v>
+      </x:c>
+      <x:c r="J18" s="27" t="n">
+        <x:v>2285.036</x:v>
+      </x:c>
+      <x:c r="K18" s="27"/>
+      <x:c r="L18" s="27"/>
+      <x:c r="M18" s="27"/>
+      <x:c r="N18" s="27"/>
+      <x:c r="O18" s="27"/>
       <x:c r="P18" s="27" t="n">
+        <x:v>1685.364</x:v>
+      </x:c>
+      <x:c r="Q18" s="27"/>
+      <x:c r="R18" s="27" t="n">
+        <x:v>1959.492</x:v>
+      </x:c>
+      <x:c r="S18" s="27" t="n">
+        <x:v>3156.973</x:v>
+      </x:c>
+      <x:c r="T18" s="27" t="n">
+        <x:v>2886.543</x:v>
+      </x:c>
+      <x:c r="U18" s="27"/>
+      <x:c r="V18" s="27"/>
+      <x:c r="W18" s="27"/>
+      <x:c r="X18" s="27"/>
+      <x:c r="Y18" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F18,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18318.604</x:v>
       </x:c>
-      <x:c r="Q18" s="27" t="n">
+      <x:c r="Z18" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F18)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R18" s="23" t="str">
+      <x:c r="AA18" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3266,39 +3425,46 @@
       <x:c r="G19" s="23" t="str">
         <x:v>查询CBN-福州晋安-东浦新村4号楼C-HRHH站点下，方位角等于90且电子下倾角不超过6的小区，返回小区名称、方位角和电子下倾角。</x:v>
       </x:c>
-      <x:c r="H19" s="23" t="str">
-        <x:v>3151.8 ms</x:v>
-      </x:c>
-      <x:c r="I19" s="23" t="str">
-        <x:v>2768.7 ms</x:v>
-      </x:c>
-      <x:c r="J19" s="23" t="str">
-        <x:v>2172.6 ms</x:v>
-      </x:c>
-      <x:c r="K19" s="23" t="str">
-        <x:v>1199.0 ms</x:v>
-      </x:c>
-      <x:c r="L19" s="23" t="str">
-        <x:v>3210.5 ms</x:v>
-      </x:c>
-      <x:c r="M19" s="23" t="str">
-        <x:v>3683.1 ms</x:v>
-      </x:c>
-      <x:c r="N19" s="23" t="str">
-        <x:v>3619.4 ms</x:v>
-      </x:c>
-      <x:c r="O19" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H19" s="27" t="n">
+        <x:v>3151.771</x:v>
+      </x:c>
+      <x:c r="I19" s="27" t="n">
+        <x:v>2768.655</x:v>
+      </x:c>
+      <x:c r="J19" s="27" t="n">
+        <x:v>2172.605</x:v>
+      </x:c>
+      <x:c r="K19" s="27"/>
+      <x:c r="L19" s="27"/>
+      <x:c r="M19" s="27"/>
+      <x:c r="N19" s="27"/>
+      <x:c r="O19" s="27"/>
       <x:c r="P19" s="27" t="n">
+        <x:v>1199.039</x:v>
+      </x:c>
+      <x:c r="Q19" s="27"/>
+      <x:c r="R19" s="27" t="n">
+        <x:v>3210.469</x:v>
+      </x:c>
+      <x:c r="S19" s="27" t="n">
+        <x:v>3683.149</x:v>
+      </x:c>
+      <x:c r="T19" s="27" t="n">
+        <x:v>3619.384</x:v>
+      </x:c>
+      <x:c r="U19" s="27"/>
+      <x:c r="V19" s="27"/>
+      <x:c r="W19" s="27"/>
+      <x:c r="X19" s="27"/>
+      <x:c r="Y19" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F19,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>19805.072</x:v>
       </x:c>
-      <x:c r="Q19" s="27" t="n">
+      <x:c r="Z19" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F19)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R19" s="23" t="str">
+      <x:c r="AA19" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3324,39 +3490,46 @@
       <x:c r="G20" s="23" t="str">
         <x:v>查询深圳东海岸三D-HRH和深圳大梅沙海滨公园D-HRW-1这两个站点下，天线高度为20或25米的小区，返回小区名称、天线高度和站点名称。</x:v>
       </x:c>
-      <x:c r="H20" s="23" t="str">
-        <x:v>2910.1 ms</x:v>
-      </x:c>
-      <x:c r="I20" s="23" t="str">
-        <x:v>2735.8 ms</x:v>
-      </x:c>
-      <x:c r="J20" s="23" t="str">
-        <x:v>2267.6 ms</x:v>
-      </x:c>
-      <x:c r="K20" s="23" t="str">
-        <x:v>1603.7 ms</x:v>
-      </x:c>
-      <x:c r="L20" s="23" t="str">
-        <x:v>2406.3 ms</x:v>
-      </x:c>
-      <x:c r="M20" s="23" t="str">
-        <x:v>3390.2 ms</x:v>
-      </x:c>
-      <x:c r="N20" s="23" t="str">
-        <x:v>3407.3 ms</x:v>
-      </x:c>
-      <x:c r="O20" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H20" s="27" t="n">
+        <x:v>2910.135</x:v>
+      </x:c>
+      <x:c r="I20" s="27" t="n">
+        <x:v>2735.842</x:v>
+      </x:c>
+      <x:c r="J20" s="27" t="n">
+        <x:v>2267.584</x:v>
+      </x:c>
+      <x:c r="K20" s="27"/>
+      <x:c r="L20" s="27"/>
+      <x:c r="M20" s="27"/>
+      <x:c r="N20" s="27"/>
+      <x:c r="O20" s="27"/>
       <x:c r="P20" s="27" t="n">
+        <x:v>1603.662</x:v>
+      </x:c>
+      <x:c r="Q20" s="27"/>
+      <x:c r="R20" s="27" t="n">
+        <x:v>2406.289</x:v>
+      </x:c>
+      <x:c r="S20" s="27" t="n">
+        <x:v>3390.234</x:v>
+      </x:c>
+      <x:c r="T20" s="27" t="n">
+        <x:v>3407.319</x:v>
+      </x:c>
+      <x:c r="U20" s="27"/>
+      <x:c r="V20" s="27"/>
+      <x:c r="W20" s="27"/>
+      <x:c r="X20" s="27"/>
+      <x:c r="Y20" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F20,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18721.065000000002</x:v>
       </x:c>
-      <x:c r="Q20" s="27" t="n">
+      <x:c r="Z20" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F20)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R20" s="23" t="str">
+      <x:c r="AA20" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3382,39 +3555,46 @@
       <x:c r="G21" s="23" t="str">
         <x:v>查询NR小区CBN-深圳大梅沙二U-H5H-0711的工程参数，包括小区名称、方位角、经度。如果该小区方位角不是180度，返回它的小区名称、方位角和经度。</x:v>
       </x:c>
-      <x:c r="H21" s="23" t="str">
-        <x:v>3443.6 ms</x:v>
-      </x:c>
-      <x:c r="I21" s="23" t="str">
-        <x:v>2734.6 ms</x:v>
-      </x:c>
-      <x:c r="J21" s="23" t="str">
-        <x:v>2014.1 ms</x:v>
-      </x:c>
-      <x:c r="K21" s="23" t="str">
-        <x:v>1652.5 ms</x:v>
-      </x:c>
-      <x:c r="L21" s="23" t="str">
-        <x:v>1819.0 ms</x:v>
-      </x:c>
-      <x:c r="M21" s="23" t="str">
-        <x:v>2507.6 ms</x:v>
-      </x:c>
-      <x:c r="N21" s="23" t="str">
-        <x:v>2907.2 ms</x:v>
-      </x:c>
-      <x:c r="O21" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H21" s="27" t="n">
+        <x:v>3443.577</x:v>
+      </x:c>
+      <x:c r="I21" s="27" t="n">
+        <x:v>2734.555</x:v>
+      </x:c>
+      <x:c r="J21" s="27" t="n">
+        <x:v>2014.112</x:v>
+      </x:c>
+      <x:c r="K21" s="27"/>
+      <x:c r="L21" s="27"/>
+      <x:c r="M21" s="27"/>
+      <x:c r="N21" s="27"/>
+      <x:c r="O21" s="27"/>
       <x:c r="P21" s="27" t="n">
+        <x:v>1652.535</x:v>
+      </x:c>
+      <x:c r="Q21" s="27"/>
+      <x:c r="R21" s="27" t="n">
+        <x:v>1818.975</x:v>
+      </x:c>
+      <x:c r="S21" s="27" t="n">
+        <x:v>2507.559</x:v>
+      </x:c>
+      <x:c r="T21" s="27" t="n">
+        <x:v>2907.194</x:v>
+      </x:c>
+      <x:c r="U21" s="27"/>
+      <x:c r="V21" s="27"/>
+      <x:c r="W21" s="27"/>
+      <x:c r="X21" s="27"/>
+      <x:c r="Y21" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F21,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>17078.506999999998</x:v>
       </x:c>
-      <x:c r="Q21" s="27" t="n">
+      <x:c r="Z21" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F21)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R21" s="23" t="str">
+      <x:c r="AA21" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3440,39 +3620,46 @@
       <x:c r="G22" s="23" t="str">
         <x:v>查询小区 CBN-福州仓山-永南路与站后路交叉口C-HRHH-515 的方位角和机械下倾角。</x:v>
       </x:c>
-      <x:c r="H22" s="23" t="str">
-        <x:v>3000.7 ms</x:v>
-      </x:c>
-      <x:c r="I22" s="23" t="str">
-        <x:v>2933.9 ms</x:v>
-      </x:c>
-      <x:c r="J22" s="23" t="str">
-        <x:v>1783.8 ms</x:v>
-      </x:c>
-      <x:c r="K22" s="23" t="str">
-        <x:v>1316.9 ms</x:v>
-      </x:c>
-      <x:c r="L22" s="23" t="str">
-        <x:v>1630.3 ms</x:v>
-      </x:c>
-      <x:c r="M22" s="23" t="str">
-        <x:v>2402.5 ms</x:v>
-      </x:c>
-      <x:c r="N22" s="23" t="str">
-        <x:v>3144.9 ms</x:v>
-      </x:c>
-      <x:c r="O22" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H22" s="27" t="n">
+        <x:v>3000.675</x:v>
+      </x:c>
+      <x:c r="I22" s="27" t="n">
+        <x:v>2933.94</x:v>
+      </x:c>
+      <x:c r="J22" s="27" t="n">
+        <x:v>1783.841</x:v>
+      </x:c>
+      <x:c r="K22" s="27"/>
+      <x:c r="L22" s="27"/>
+      <x:c r="M22" s="27"/>
+      <x:c r="N22" s="27"/>
+      <x:c r="O22" s="27"/>
       <x:c r="P22" s="27" t="n">
+        <x:v>1316.891</x:v>
+      </x:c>
+      <x:c r="Q22" s="27"/>
+      <x:c r="R22" s="27" t="n">
+        <x:v>1630.316</x:v>
+      </x:c>
+      <x:c r="S22" s="27" t="n">
+        <x:v>2402.541</x:v>
+      </x:c>
+      <x:c r="T22" s="27" t="n">
+        <x:v>3144.932</x:v>
+      </x:c>
+      <x:c r="U22" s="27"/>
+      <x:c r="V22" s="27"/>
+      <x:c r="W22" s="27"/>
+      <x:c r="X22" s="27"/>
+      <x:c r="Y22" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F22,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>16213.136000000002</x:v>
       </x:c>
-      <x:c r="Q22" s="27" t="n">
+      <x:c r="Z22" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F22)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R22" s="23" t="str">
+      <x:c r="AA22" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3498,39 +3685,46 @@
       <x:c r="G23" s="23" t="str">
         <x:v>查询深圳大梅沙D-HRH站点下所有小区的经度和纬度</x:v>
       </x:c>
-      <x:c r="H23" s="23" t="str">
-        <x:v>2872.7 ms</x:v>
-      </x:c>
-      <x:c r="I23" s="23" t="str">
-        <x:v>2572.5 ms</x:v>
-      </x:c>
-      <x:c r="J23" s="23" t="str">
-        <x:v>1428.7 ms</x:v>
-      </x:c>
-      <x:c r="K23" s="23" t="str">
-        <x:v>1186.3 ms</x:v>
-      </x:c>
-      <x:c r="L23" s="23" t="str">
-        <x:v>1446.4 ms</x:v>
-      </x:c>
-      <x:c r="M23" s="23" t="str">
-        <x:v>2019.5 ms</x:v>
-      </x:c>
-      <x:c r="N23" s="23" t="str">
-        <x:v>2831.6 ms</x:v>
-      </x:c>
-      <x:c r="O23" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H23" s="27" t="n">
+        <x:v>2872.697</x:v>
+      </x:c>
+      <x:c r="I23" s="27" t="n">
+        <x:v>2572.546</x:v>
+      </x:c>
+      <x:c r="J23" s="27" t="n">
+        <x:v>1428.663</x:v>
+      </x:c>
+      <x:c r="K23" s="27"/>
+      <x:c r="L23" s="27"/>
+      <x:c r="M23" s="27"/>
+      <x:c r="N23" s="27"/>
+      <x:c r="O23" s="27"/>
       <x:c r="P23" s="27" t="n">
+        <x:v>1186.348</x:v>
+      </x:c>
+      <x:c r="Q23" s="27"/>
+      <x:c r="R23" s="27" t="n">
+        <x:v>1446.383</x:v>
+      </x:c>
+      <x:c r="S23" s="27" t="n">
+        <x:v>2019.502</x:v>
+      </x:c>
+      <x:c r="T23" s="27" t="n">
+        <x:v>2831.554</x:v>
+      </x:c>
+      <x:c r="U23" s="27"/>
+      <x:c r="V23" s="27"/>
+      <x:c r="W23" s="27"/>
+      <x:c r="X23" s="27"/>
+      <x:c r="Y23" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F23,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>14357.693000000001</x:v>
       </x:c>
-      <x:c r="Q23" s="27" t="n">
+      <x:c r="Z23" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F23)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R23" s="23" t="str">
+      <x:c r="AA23" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3556,39 +3750,46 @@
       <x:c r="G24" s="23" t="str">
         <x:v>查询小区 CBN-深圳东华风车U-H5H-0711 的基站标识和小区名称。</x:v>
       </x:c>
-      <x:c r="H24" s="23" t="str">
-        <x:v>2842.6 ms</x:v>
-      </x:c>
-      <x:c r="I24" s="23" t="str">
-        <x:v>2570.7 ms</x:v>
-      </x:c>
-      <x:c r="J24" s="23" t="str">
-        <x:v>1601.5 ms</x:v>
-      </x:c>
-      <x:c r="K24" s="23" t="str">
-        <x:v>1307.6 ms</x:v>
-      </x:c>
-      <x:c r="L24" s="23" t="str">
-        <x:v>1642.4 ms</x:v>
-      </x:c>
-      <x:c r="M24" s="23" t="str">
-        <x:v>2210.1 ms</x:v>
-      </x:c>
-      <x:c r="N24" s="23" t="str">
-        <x:v>3147.2 ms</x:v>
-      </x:c>
-      <x:c r="O24" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H24" s="27" t="n">
+        <x:v>2842.632</x:v>
+      </x:c>
+      <x:c r="I24" s="27" t="n">
+        <x:v>2570.748</x:v>
+      </x:c>
+      <x:c r="J24" s="27" t="n">
+        <x:v>1601.481</x:v>
+      </x:c>
+      <x:c r="K24" s="27"/>
+      <x:c r="L24" s="27"/>
+      <x:c r="M24" s="27"/>
+      <x:c r="N24" s="27"/>
+      <x:c r="O24" s="27"/>
       <x:c r="P24" s="27" t="n">
+        <x:v>1307.56</x:v>
+      </x:c>
+      <x:c r="Q24" s="27"/>
+      <x:c r="R24" s="27" t="n">
+        <x:v>1642.444</x:v>
+      </x:c>
+      <x:c r="S24" s="27" t="n">
+        <x:v>2210.127</x:v>
+      </x:c>
+      <x:c r="T24" s="27" t="n">
+        <x:v>3147.178</x:v>
+      </x:c>
+      <x:c r="U24" s="27"/>
+      <x:c r="V24" s="27"/>
+      <x:c r="W24" s="27"/>
+      <x:c r="X24" s="27"/>
+      <x:c r="Y24" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F24,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>15322.17</x:v>
       </x:c>
-      <x:c r="Q24" s="27" t="n">
+      <x:c r="Z24" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F24)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R24" s="23" t="str">
+      <x:c r="AA24" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3614,39 +3815,40 @@
       <x:c r="G25" s="23" t="str">
         <x:v>查询小区 CBN-福州晋安-福厦高铁鼓山鼓一隧道C-HRRH-513 的方向角。</x:v>
       </x:c>
-      <x:c r="H25" s="23" t="str">
-        <x:v>2662.3 ms</x:v>
-      </x:c>
-      <x:c r="I25" s="23" t="str">
-        <x:v>2610.0 ms</x:v>
-      </x:c>
-      <x:c r="J25" s="23" t="str">
-        <x:v>2099.7 ms</x:v>
-      </x:c>
-      <x:c r="K25" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="L25" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="M25" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="N25" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="O25" s="23" t="str">
-        <x:v>AskUserQuestion: 3034.1 ms</x:v>
-      </x:c>
-      <x:c r="P25" s="27" t="n">
+      <x:c r="H25" s="27" t="n">
+        <x:v>2662.278</x:v>
+      </x:c>
+      <x:c r="I25" s="27" t="n">
+        <x:v>2609.982</x:v>
+      </x:c>
+      <x:c r="J25" s="27" t="n">
+        <x:v>2099.695</x:v>
+      </x:c>
+      <x:c r="K25" s="27"/>
+      <x:c r="L25" s="27"/>
+      <x:c r="M25" s="27"/>
+      <x:c r="N25" s="27"/>
+      <x:c r="O25" s="27"/>
+      <x:c r="P25" s="27"/>
+      <x:c r="Q25" s="27"/>
+      <x:c r="R25" s="27"/>
+      <x:c r="S25" s="27"/>
+      <x:c r="T25" s="27"/>
+      <x:c r="U25" s="27" t="n">
+        <x:v>3034.064</x:v>
+      </x:c>
+      <x:c r="V25" s="27"/>
+      <x:c r="W25" s="27"/>
+      <x:c r="X25" s="27"/>
+      <x:c r="Y25" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F25,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>10406.019</x:v>
       </x:c>
-      <x:c r="Q25" s="27" t="n">
+      <x:c r="Z25" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F25)</x:f>
         <x:v>4</x:v>
       </x:c>
-      <x:c r="R25" s="23" t="str">
+      <x:c r="AA25" s="23" t="str">
         <x:v>缺少：Recipe - Qwen总结、AICO总结、问题推荐</x:v>
       </x:c>
     </x:row>
@@ -3672,39 +3874,46 @@
       <x:c r="G26" s="23" t="str">
         <x:v>查询站点 CBN-深圳梅沙湾U-H5H 下所有小区的站点名称、方位角和机械下倾角</x:v>
       </x:c>
-      <x:c r="H26" s="23" t="str">
-        <x:v>2740.3 ms</x:v>
-      </x:c>
-      <x:c r="I26" s="23" t="str">
-        <x:v>2711.8 ms</x:v>
-      </x:c>
-      <x:c r="J26" s="23" t="str">
-        <x:v>1637.0 ms</x:v>
-      </x:c>
-      <x:c r="K26" s="23" t="str">
-        <x:v>1274.8 ms</x:v>
-      </x:c>
-      <x:c r="L26" s="23" t="str">
-        <x:v>2788.2 ms</x:v>
-      </x:c>
-      <x:c r="M26" s="23" t="str">
-        <x:v>3290.4 ms</x:v>
-      </x:c>
-      <x:c r="N26" s="23" t="str">
-        <x:v>3317.9 ms</x:v>
-      </x:c>
-      <x:c r="O26" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H26" s="27" t="n">
+        <x:v>2740.349</x:v>
+      </x:c>
+      <x:c r="I26" s="27" t="n">
+        <x:v>2711.815</x:v>
+      </x:c>
+      <x:c r="J26" s="27" t="n">
+        <x:v>1637</x:v>
+      </x:c>
+      <x:c r="K26" s="27"/>
+      <x:c r="L26" s="27"/>
+      <x:c r="M26" s="27"/>
+      <x:c r="N26" s="27"/>
+      <x:c r="O26" s="27"/>
       <x:c r="P26" s="27" t="n">
+        <x:v>1274.791</x:v>
+      </x:c>
+      <x:c r="Q26" s="27"/>
+      <x:c r="R26" s="27" t="n">
+        <x:v>2788.228</x:v>
+      </x:c>
+      <x:c r="S26" s="27" t="n">
+        <x:v>3290.357</x:v>
+      </x:c>
+      <x:c r="T26" s="27" t="n">
+        <x:v>3317.923</x:v>
+      </x:c>
+      <x:c r="U26" s="27"/>
+      <x:c r="V26" s="27"/>
+      <x:c r="W26" s="27"/>
+      <x:c r="X26" s="27"/>
+      <x:c r="Y26" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F26,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>17760.463</x:v>
       </x:c>
-      <x:c r="Q26" s="27" t="n">
+      <x:c r="Z26" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F26)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R26" s="23" t="str">
+      <x:c r="AA26" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3730,39 +3939,46 @@
       <x:c r="G27" s="23" t="str">
         <x:v>查询小区 CBN-福州仓山-火车南站西广场南侧高架桥旁C-HRHH-513 和 CBN-福州晋安-站东路三环北路交叉西C-HRRH-512 的经度、纬度和方位角。</x:v>
       </x:c>
-      <x:c r="H27" s="23" t="str">
-        <x:v>3393.8 ms</x:v>
-      </x:c>
-      <x:c r="I27" s="23" t="str">
-        <x:v>3219.3 ms</x:v>
-      </x:c>
-      <x:c r="J27" s="23" t="str">
-        <x:v>2116.7 ms</x:v>
-      </x:c>
-      <x:c r="K27" s="23" t="str">
-        <x:v>1769.3 ms</x:v>
-      </x:c>
-      <x:c r="L27" s="23" t="str">
-        <x:v>2210.3 ms</x:v>
-      </x:c>
-      <x:c r="M27" s="23" t="str">
-        <x:v>2838.6 ms</x:v>
-      </x:c>
-      <x:c r="N27" s="23" t="str">
-        <x:v>3712.7 ms</x:v>
-      </x:c>
-      <x:c r="O27" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H27" s="27" t="n">
+        <x:v>3393.783</x:v>
+      </x:c>
+      <x:c r="I27" s="27" t="n">
+        <x:v>3219.279</x:v>
+      </x:c>
+      <x:c r="J27" s="27" t="n">
+        <x:v>2116.668</x:v>
+      </x:c>
+      <x:c r="K27" s="27"/>
+      <x:c r="L27" s="27"/>
+      <x:c r="M27" s="27"/>
+      <x:c r="N27" s="27"/>
+      <x:c r="O27" s="27"/>
       <x:c r="P27" s="27" t="n">
+        <x:v>1769.341</x:v>
+      </x:c>
+      <x:c r="Q27" s="27"/>
+      <x:c r="R27" s="27" t="n">
+        <x:v>2210.271</x:v>
+      </x:c>
+      <x:c r="S27" s="27" t="n">
+        <x:v>2838.573</x:v>
+      </x:c>
+      <x:c r="T27" s="27" t="n">
+        <x:v>3712.748</x:v>
+      </x:c>
+      <x:c r="U27" s="27"/>
+      <x:c r="V27" s="27"/>
+      <x:c r="W27" s="27"/>
+      <x:c r="X27" s="27"/>
+      <x:c r="Y27" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F27,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>19260.663</x:v>
       </x:c>
-      <x:c r="Q27" s="27" t="n">
+      <x:c r="Z27" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F27)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R27" s="23" t="str">
+      <x:c r="AA27" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3788,39 +4004,46 @@
       <x:c r="G28" s="23" t="str">
         <x:v>查询深圳奥特莱斯D-HRH和深圳上威梅沙二D-HRH两个站点下所有小区的天线高度和电子下倾角。</x:v>
       </x:c>
-      <x:c r="H28" s="23" t="str">
-        <x:v>3351.0 ms</x:v>
-      </x:c>
-      <x:c r="I28" s="23" t="str">
-        <x:v>3074.6 ms</x:v>
-      </x:c>
-      <x:c r="J28" s="23" t="str">
-        <x:v>1789.2 ms</x:v>
-      </x:c>
-      <x:c r="K28" s="23" t="str">
-        <x:v>1291.9 ms</x:v>
-      </x:c>
-      <x:c r="L28" s="23" t="str">
-        <x:v>2135.6 ms</x:v>
-      </x:c>
-      <x:c r="M28" s="23" t="str">
-        <x:v>3229.9 ms</x:v>
-      </x:c>
-      <x:c r="N28" s="23" t="str">
-        <x:v>3801.2 ms</x:v>
-      </x:c>
-      <x:c r="O28" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H28" s="27" t="n">
+        <x:v>3350.982</x:v>
+      </x:c>
+      <x:c r="I28" s="27" t="n">
+        <x:v>3074.568</x:v>
+      </x:c>
+      <x:c r="J28" s="27" t="n">
+        <x:v>1789.192</x:v>
+      </x:c>
+      <x:c r="K28" s="27"/>
+      <x:c r="L28" s="27"/>
+      <x:c r="M28" s="27"/>
+      <x:c r="N28" s="27"/>
+      <x:c r="O28" s="27"/>
       <x:c r="P28" s="27" t="n">
+        <x:v>1291.885</x:v>
+      </x:c>
+      <x:c r="Q28" s="27"/>
+      <x:c r="R28" s="27" t="n">
+        <x:v>2135.637</x:v>
+      </x:c>
+      <x:c r="S28" s="27" t="n">
+        <x:v>3229.885</x:v>
+      </x:c>
+      <x:c r="T28" s="27" t="n">
+        <x:v>3801.16</x:v>
+      </x:c>
+      <x:c r="U28" s="27"/>
+      <x:c r="V28" s="27"/>
+      <x:c r="W28" s="27"/>
+      <x:c r="X28" s="27"/>
+      <x:c r="Y28" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F28,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18673.309</x:v>
       </x:c>
-      <x:c r="Q28" s="27" t="n">
+      <x:c r="Z28" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F28)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R28" s="23" t="str">
+      <x:c r="AA28" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3846,39 +4069,46 @@
       <x:c r="G29" s="23" t="str">
         <x:v>查询小区 CBN-深圳大梅沙二U-H5H-0711、CBN-深圳盐梅路一U-H5H-0712 和 CBN-深圳东海岸三[CBN-深圳天麓八区U-H5H]U-H5H-0711 这三个小区的站点名称。</x:v>
       </x:c>
-      <x:c r="H29" s="23" t="str">
-        <x:v>3513.1 ms</x:v>
-      </x:c>
-      <x:c r="I29" s="23" t="str">
-        <x:v>2891.7 ms</x:v>
-      </x:c>
-      <x:c r="J29" s="23" t="str">
-        <x:v>2108.6 ms</x:v>
-      </x:c>
-      <x:c r="K29" s="23" t="str">
-        <x:v>1889.3 ms</x:v>
-      </x:c>
-      <x:c r="L29" s="23" t="str">
-        <x:v>2543.4 ms</x:v>
-      </x:c>
-      <x:c r="M29" s="23" t="str">
-        <x:v>3150.0 ms</x:v>
-      </x:c>
-      <x:c r="N29" s="23" t="str">
-        <x:v>3045.0 ms</x:v>
-      </x:c>
-      <x:c r="O29" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H29" s="27" t="n">
+        <x:v>3513.104</x:v>
+      </x:c>
+      <x:c r="I29" s="27" t="n">
+        <x:v>2891.715</x:v>
+      </x:c>
+      <x:c r="J29" s="27" t="n">
+        <x:v>2108.59</x:v>
+      </x:c>
+      <x:c r="K29" s="27"/>
+      <x:c r="L29" s="27"/>
+      <x:c r="M29" s="27"/>
+      <x:c r="N29" s="27"/>
+      <x:c r="O29" s="27"/>
       <x:c r="P29" s="27" t="n">
+        <x:v>1889.295</x:v>
+      </x:c>
+      <x:c r="Q29" s="27"/>
+      <x:c r="R29" s="27" t="n">
+        <x:v>2543.366</x:v>
+      </x:c>
+      <x:c r="S29" s="27" t="n">
+        <x:v>3150.014</x:v>
+      </x:c>
+      <x:c r="T29" s="27" t="n">
+        <x:v>3044.96</x:v>
+      </x:c>
+      <x:c r="U29" s="27"/>
+      <x:c r="V29" s="27"/>
+      <x:c r="W29" s="27"/>
+      <x:c r="X29" s="27"/>
+      <x:c r="Y29" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F29,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>19141.043999999998</x:v>
       </x:c>
-      <x:c r="Q29" s="27" t="n">
+      <x:c r="Z29" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F29)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R29" s="23" t="str">
+      <x:c r="AA29" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3904,39 +4134,48 @@
       <x:c r="G30" s="23" t="str">
         <x:v>对比一下 CBN-福州晋安-东浦新村4号楼C-HRHH-513 和 CBN-福州晋安-东浦新村4号楼C-HRHH-514 这两个小区的设备厂商和小区名称。</x:v>
       </x:c>
-      <x:c r="H30" s="23" t="str">
-        <x:v>2883.5 ms</x:v>
-      </x:c>
-      <x:c r="I30" s="23" t="str">
-        <x:v>2771.8 ms</x:v>
-      </x:c>
-      <x:c r="J30" s="23" t="str">
-        <x:v>1907.5 ms</x:v>
-      </x:c>
-      <x:c r="K30" s="23" t="str">
-        <x:v>第1次 1680.6 ms；第2次 2422.0 ms</x:v>
-      </x:c>
-      <x:c r="L30" s="23" t="str">
-        <x:v>2846.5 ms</x:v>
-      </x:c>
-      <x:c r="M30" s="23" t="str">
-        <x:v>3918.2 ms</x:v>
-      </x:c>
-      <x:c r="N30" s="23" t="str">
-        <x:v>3493.4 ms</x:v>
-      </x:c>
-      <x:c r="O30" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H30" s="27" t="n">
+        <x:v>2883.487</x:v>
+      </x:c>
+      <x:c r="I30" s="27" t="n">
+        <x:v>2771.772</x:v>
+      </x:c>
+      <x:c r="J30" s="27" t="n">
+        <x:v>1907.463</x:v>
+      </x:c>
+      <x:c r="K30" s="27"/>
+      <x:c r="L30" s="27"/>
+      <x:c r="M30" s="27"/>
+      <x:c r="N30" s="27"/>
+      <x:c r="O30" s="27"/>
       <x:c r="P30" s="27" t="n">
+        <x:v>1680.605</x:v>
+      </x:c>
+      <x:c r="Q30" s="27" t="n">
+        <x:v>2421.991</x:v>
+      </x:c>
+      <x:c r="R30" s="27" t="n">
+        <x:v>2846.494</x:v>
+      </x:c>
+      <x:c r="S30" s="27" t="n">
+        <x:v>3918.151</x:v>
+      </x:c>
+      <x:c r="T30" s="27" t="n">
+        <x:v>3493.396</x:v>
+      </x:c>
+      <x:c r="U30" s="27"/>
+      <x:c r="V30" s="27"/>
+      <x:c r="W30" s="27"/>
+      <x:c r="X30" s="27"/>
+      <x:c r="Y30" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F30,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>21923.359</x:v>
       </x:c>
-      <x:c r="Q30" s="27" t="n">
+      <x:c r="Z30" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F30)</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="R30" s="23" t="str">
+      <x:c r="AA30" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -3962,39 +4201,46 @@
       <x:c r="G31" s="23" t="str">
         <x:v>查询站点 CBN-福州仓山-福州南站火车南站西北美化塔C-HRRH 和 CBN-深圳大梅沙U-H5H 下所有小区的方位角和天线高度。</x:v>
       </x:c>
-      <x:c r="H31" s="23" t="str">
-        <x:v>3318.2 ms</x:v>
-      </x:c>
-      <x:c r="I31" s="23" t="str">
-        <x:v>2900.8 ms</x:v>
-      </x:c>
-      <x:c r="J31" s="23" t="str">
-        <x:v>1927.2 ms</x:v>
-      </x:c>
-      <x:c r="K31" s="23" t="str">
-        <x:v>1521.9 ms</x:v>
-      </x:c>
-      <x:c r="L31" s="23" t="str">
-        <x:v>2783.3 ms</x:v>
-      </x:c>
-      <x:c r="M31" s="23" t="str">
-        <x:v>3235.4 ms</x:v>
-      </x:c>
-      <x:c r="N31" s="23" t="str">
-        <x:v>3087.7 ms</x:v>
-      </x:c>
-      <x:c r="O31" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H31" s="27" t="n">
+        <x:v>3318.185</x:v>
+      </x:c>
+      <x:c r="I31" s="27" t="n">
+        <x:v>2900.821</x:v>
+      </x:c>
+      <x:c r="J31" s="27" t="n">
+        <x:v>1927.23</x:v>
+      </x:c>
+      <x:c r="K31" s="27"/>
+      <x:c r="L31" s="27"/>
+      <x:c r="M31" s="27"/>
+      <x:c r="N31" s="27"/>
+      <x:c r="O31" s="27"/>
       <x:c r="P31" s="27" t="n">
+        <x:v>1521.892</x:v>
+      </x:c>
+      <x:c r="Q31" s="27"/>
+      <x:c r="R31" s="27" t="n">
+        <x:v>2783.347</x:v>
+      </x:c>
+      <x:c r="S31" s="27" t="n">
+        <x:v>3235.416</x:v>
+      </x:c>
+      <x:c r="T31" s="27" t="n">
+        <x:v>3087.721</x:v>
+      </x:c>
+      <x:c r="U31" s="27"/>
+      <x:c r="V31" s="27"/>
+      <x:c r="W31" s="27"/>
+      <x:c r="X31" s="27"/>
+      <x:c r="Y31" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F31,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18774.612</x:v>
       </x:c>
-      <x:c r="Q31" s="27" t="n">
+      <x:c r="Z31" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F31)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R31" s="23" t="str">
+      <x:c r="AA31" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4020,39 +4266,46 @@
       <x:c r="G32" s="23" t="str">
         <x:v>查询深圳大梅沙D-HRH站点下5G小区的小区名称和方位角。</x:v>
       </x:c>
-      <x:c r="H32" s="23" t="str">
-        <x:v>2921.5 ms</x:v>
-      </x:c>
-      <x:c r="I32" s="23" t="str">
-        <x:v>2716.5 ms</x:v>
-      </x:c>
-      <x:c r="J32" s="23" t="str">
-        <x:v>1523.2 ms</x:v>
-      </x:c>
-      <x:c r="K32" s="23" t="str">
-        <x:v>1297.1 ms</x:v>
-      </x:c>
-      <x:c r="L32" s="23" t="str">
-        <x:v>1758.0 ms</x:v>
-      </x:c>
-      <x:c r="M32" s="23" t="str">
-        <x:v>2763.0 ms</x:v>
-      </x:c>
-      <x:c r="N32" s="23" t="str">
-        <x:v>3290.4 ms</x:v>
-      </x:c>
-      <x:c r="O32" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H32" s="27" t="n">
+        <x:v>2921.537</x:v>
+      </x:c>
+      <x:c r="I32" s="27" t="n">
+        <x:v>2716.489</x:v>
+      </x:c>
+      <x:c r="J32" s="27" t="n">
+        <x:v>1523.225</x:v>
+      </x:c>
+      <x:c r="K32" s="27"/>
+      <x:c r="L32" s="27"/>
+      <x:c r="M32" s="27"/>
+      <x:c r="N32" s="27"/>
+      <x:c r="O32" s="27"/>
       <x:c r="P32" s="27" t="n">
+        <x:v>1297.122</x:v>
+      </x:c>
+      <x:c r="Q32" s="27"/>
+      <x:c r="R32" s="27" t="n">
+        <x:v>1758.008</x:v>
+      </x:c>
+      <x:c r="S32" s="27" t="n">
+        <x:v>2763.008</x:v>
+      </x:c>
+      <x:c r="T32" s="27" t="n">
+        <x:v>3290.448</x:v>
+      </x:c>
+      <x:c r="U32" s="27"/>
+      <x:c r="V32" s="27"/>
+      <x:c r="W32" s="27"/>
+      <x:c r="X32" s="27"/>
+      <x:c r="Y32" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F32,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>16269.837</x:v>
       </x:c>
-      <x:c r="Q32" s="27" t="n">
+      <x:c r="Z32" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F32)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R32" s="23" t="str">
+      <x:c r="AA32" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4078,39 +4331,46 @@
       <x:c r="G33" s="23" t="str">
         <x:v>查询CBN-深圳大梅沙二U-H5H-0712这个NR小区的机械下倾角和电子下倾角</x:v>
       </x:c>
-      <x:c r="H33" s="23" t="str">
-        <x:v>2671.4 ms</x:v>
-      </x:c>
-      <x:c r="I33" s="23" t="str">
-        <x:v>2708.3 ms</x:v>
-      </x:c>
-      <x:c r="J33" s="23" t="str">
-        <x:v>1617.3 ms</x:v>
-      </x:c>
-      <x:c r="K33" s="23" t="str">
-        <x:v>1417.2 ms</x:v>
-      </x:c>
-      <x:c r="L33" s="23" t="str">
-        <x:v>1500.1 ms</x:v>
-      </x:c>
-      <x:c r="M33" s="23" t="str">
-        <x:v>2100.8 ms</x:v>
-      </x:c>
-      <x:c r="N33" s="23" t="str">
-        <x:v>2664.8 ms</x:v>
-      </x:c>
-      <x:c r="O33" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H33" s="27" t="n">
+        <x:v>2671.376</x:v>
+      </x:c>
+      <x:c r="I33" s="27" t="n">
+        <x:v>2708.276</x:v>
+      </x:c>
+      <x:c r="J33" s="27" t="n">
+        <x:v>1617.35</x:v>
+      </x:c>
+      <x:c r="K33" s="27"/>
+      <x:c r="L33" s="27"/>
+      <x:c r="M33" s="27"/>
+      <x:c r="N33" s="27"/>
+      <x:c r="O33" s="27"/>
       <x:c r="P33" s="27" t="n">
+        <x:v>1417.199</x:v>
+      </x:c>
+      <x:c r="Q33" s="27"/>
+      <x:c r="R33" s="27" t="n">
+        <x:v>1500.11</x:v>
+      </x:c>
+      <x:c r="S33" s="27" t="n">
+        <x:v>2100.799</x:v>
+      </x:c>
+      <x:c r="T33" s="27" t="n">
+        <x:v>2664.833</x:v>
+      </x:c>
+      <x:c r="U33" s="27"/>
+      <x:c r="V33" s="27"/>
+      <x:c r="W33" s="27"/>
+      <x:c r="X33" s="27"/>
+      <x:c r="Y33" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F33,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>14679.943000000001</x:v>
       </x:c>
-      <x:c r="Q33" s="27" t="n">
+      <x:c r="Z33" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F33)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R33" s="23" t="str">
+      <x:c r="AA33" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4136,39 +4396,48 @@
       <x:c r="G34" s="23" t="str">
         <x:v>查询深圳奥特莱斯D-HRH和深圳梅沙湾二D-HRH这两个站点下5G小区的站点名称、经度和纬度。</x:v>
       </x:c>
-      <x:c r="H34" s="23" t="str">
-        <x:v>2874.3 ms</x:v>
-      </x:c>
-      <x:c r="I34" s="23" t="str">
-        <x:v>2654.9 ms</x:v>
-      </x:c>
-      <x:c r="J34" s="23" t="str">
-        <x:v>1602.2 ms</x:v>
-      </x:c>
-      <x:c r="K34" s="23" t="str">
-        <x:v>第1次 1284.8 ms；第2次 1586.1 ms</x:v>
-      </x:c>
-      <x:c r="L34" s="23" t="str">
-        <x:v>3856.6 ms</x:v>
-      </x:c>
-      <x:c r="M34" s="23" t="str">
-        <x:v>3535.4 ms</x:v>
-      </x:c>
-      <x:c r="N34" s="23" t="str">
-        <x:v>3257.5 ms</x:v>
-      </x:c>
-      <x:c r="O34" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H34" s="27" t="n">
+        <x:v>2874.286</x:v>
+      </x:c>
+      <x:c r="I34" s="27" t="n">
+        <x:v>2654.872</x:v>
+      </x:c>
+      <x:c r="J34" s="27" t="n">
+        <x:v>1602.209</x:v>
+      </x:c>
+      <x:c r="K34" s="27"/>
+      <x:c r="L34" s="27"/>
+      <x:c r="M34" s="27"/>
+      <x:c r="N34" s="27"/>
+      <x:c r="O34" s="27"/>
       <x:c r="P34" s="27" t="n">
+        <x:v>1284.818</x:v>
+      </x:c>
+      <x:c r="Q34" s="27" t="n">
+        <x:v>1586.145</x:v>
+      </x:c>
+      <x:c r="R34" s="27" t="n">
+        <x:v>3856.616</x:v>
+      </x:c>
+      <x:c r="S34" s="27" t="n">
+        <x:v>3535.447</x:v>
+      </x:c>
+      <x:c r="T34" s="27" t="n">
+        <x:v>3257.523</x:v>
+      </x:c>
+      <x:c r="U34" s="27"/>
+      <x:c r="V34" s="27"/>
+      <x:c r="W34" s="27"/>
+      <x:c r="X34" s="27"/>
+      <x:c r="Y34" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F34,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>20651.916</x:v>
       </x:c>
-      <x:c r="Q34" s="27" t="n">
+      <x:c r="Z34" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F34)</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="R34" s="23" t="str">
+      <x:c r="AA34" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4194,39 +4463,46 @@
       <x:c r="G35" s="23" t="str">
         <x:v>查询5G小区 CBN-福州仓山-福州火车南站C-HRHH-521 的小区标识（Cell ID）和移动网号（MNC）。</x:v>
       </x:c>
-      <x:c r="H35" s="23" t="str">
-        <x:v>4488.0 ms</x:v>
-      </x:c>
-      <x:c r="I35" s="23" t="str">
-        <x:v>13963.6 ms</x:v>
-      </x:c>
-      <x:c r="J35" s="23" t="str">
-        <x:v>14196.8 ms</x:v>
-      </x:c>
-      <x:c r="K35" s="23" t="str">
-        <x:v>1275.9 ms</x:v>
-      </x:c>
-      <x:c r="L35" s="23" t="str">
-        <x:v>1753.6 ms</x:v>
-      </x:c>
-      <x:c r="M35" s="23" t="str">
-        <x:v>17957.8 ms</x:v>
-      </x:c>
-      <x:c r="N35" s="23" t="str">
-        <x:v>9918.9 ms</x:v>
-      </x:c>
-      <x:c r="O35" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H35" s="27" t="n">
+        <x:v>4487.988</x:v>
+      </x:c>
+      <x:c r="I35" s="27" t="n">
+        <x:v>13963.612</x:v>
+      </x:c>
+      <x:c r="J35" s="27" t="n">
+        <x:v>14196.817</x:v>
+      </x:c>
+      <x:c r="K35" s="27"/>
+      <x:c r="L35" s="27"/>
+      <x:c r="M35" s="27"/>
+      <x:c r="N35" s="27"/>
+      <x:c r="O35" s="27"/>
       <x:c r="P35" s="27" t="n">
+        <x:v>1275.921</x:v>
+      </x:c>
+      <x:c r="Q35" s="27"/>
+      <x:c r="R35" s="27" t="n">
+        <x:v>1753.582</x:v>
+      </x:c>
+      <x:c r="S35" s="27" t="n">
+        <x:v>17957.763</x:v>
+      </x:c>
+      <x:c r="T35" s="27" t="n">
+        <x:v>9918.948</x:v>
+      </x:c>
+      <x:c r="U35" s="27"/>
+      <x:c r="V35" s="27"/>
+      <x:c r="W35" s="27"/>
+      <x:c r="X35" s="27"/>
+      <x:c r="Y35" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F35,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>63554.630999999994</x:v>
       </x:c>
-      <x:c r="Q35" s="27" t="n">
+      <x:c r="Z35" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F35)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R35" s="23" t="str">
+      <x:c r="AA35" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4252,39 +4528,46 @@
       <x:c r="G36" s="23" t="str">
         <x:v>查询CBN-深圳上威梅沙二U-H5H-0711和CBN-深圳东华风车U-H5H-0711这两个NR小区的方向角和天线高度。</x:v>
       </x:c>
-      <x:c r="H36" s="23" t="str">
-        <x:v>17286.7 ms</x:v>
-      </x:c>
-      <x:c r="I36" s="23" t="str">
-        <x:v>20770.8 ms</x:v>
-      </x:c>
-      <x:c r="J36" s="23" t="str">
-        <x:v>24036.1 ms</x:v>
-      </x:c>
-      <x:c r="K36" s="23" t="str">
-        <x:v>1830.3 ms</x:v>
-      </x:c>
-      <x:c r="L36" s="23" t="str">
-        <x:v>1640.8 ms</x:v>
-      </x:c>
-      <x:c r="M36" s="23" t="str">
-        <x:v>9576.6 ms</x:v>
-      </x:c>
-      <x:c r="N36" s="23" t="str">
-        <x:v>21049.9 ms</x:v>
-      </x:c>
-      <x:c r="O36" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H36" s="27" t="n">
+        <x:v>17286.739</x:v>
+      </x:c>
+      <x:c r="I36" s="27" t="n">
+        <x:v>20770.793</x:v>
+      </x:c>
+      <x:c r="J36" s="27" t="n">
+        <x:v>24036.115</x:v>
+      </x:c>
+      <x:c r="K36" s="27"/>
+      <x:c r="L36" s="27"/>
+      <x:c r="M36" s="27"/>
+      <x:c r="N36" s="27"/>
+      <x:c r="O36" s="27"/>
       <x:c r="P36" s="27" t="n">
+        <x:v>1830.289</x:v>
+      </x:c>
+      <x:c r="Q36" s="27"/>
+      <x:c r="R36" s="27" t="n">
+        <x:v>1640.796</x:v>
+      </x:c>
+      <x:c r="S36" s="27" t="n">
+        <x:v>9576.58</x:v>
+      </x:c>
+      <x:c r="T36" s="27" t="n">
+        <x:v>21049.916</x:v>
+      </x:c>
+      <x:c r="U36" s="27"/>
+      <x:c r="V36" s="27"/>
+      <x:c r="W36" s="27"/>
+      <x:c r="X36" s="27"/>
+      <x:c r="Y36" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F36,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>96191.228</x:v>
       </x:c>
-      <x:c r="Q36" s="27" t="n">
+      <x:c r="Z36" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F36)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R36" s="23" t="str">
+      <x:c r="AA36" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4310,39 +4593,56 @@
       <x:c r="G37" s="23" t="str">
         <x:v>查询深圳大梅沙海滨公园D-HRW站点下，天线高度超过30米的小区，返回小区名称、天线高度和方位角。</x:v>
       </x:c>
-      <x:c r="H37" s="23" t="str">
-        <x:v>20074.0 ms</x:v>
-      </x:c>
-      <x:c r="I37" s="23" t="str">
-        <x:v>26821.0 ms</x:v>
-      </x:c>
-      <x:c r="J37" s="23" t="str">
-        <x:v>第1次 31259.0 ms；第2次 2547.1 ms；第3次 13142.9 ms；第4次 13989.2 ms；第5次 2576.4 ms；第6次 30091.7 ms</x:v>
-      </x:c>
-      <x:c r="K37" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="L37" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="M37" s="23" t="str">
-        <x:v>17210.4 ms</x:v>
-      </x:c>
-      <x:c r="N37" s="23" t="str">
-        <x:v>15695.8 ms</x:v>
-      </x:c>
-      <x:c r="O37" s="23" t="str">
-        <x:v>第1次 ToolSearch: 4932.3 ms；第2次 Agent: 3944.4 ms</x:v>
-      </x:c>
-      <x:c r="P37" s="27" t="n">
+      <x:c r="H37" s="27" t="n">
+        <x:v>20073.974</x:v>
+      </x:c>
+      <x:c r="I37" s="27" t="n">
+        <x:v>26820.954</x:v>
+      </x:c>
+      <x:c r="J37" s="27" t="n">
+        <x:v>31259.046</x:v>
+      </x:c>
+      <x:c r="K37" s="27" t="n">
+        <x:v>2547.105</x:v>
+      </x:c>
+      <x:c r="L37" s="27" t="n">
+        <x:v>13142.917</x:v>
+      </x:c>
+      <x:c r="M37" s="27" t="n">
+        <x:v>13989.18</x:v>
+      </x:c>
+      <x:c r="N37" s="27" t="n">
+        <x:v>2576.352</x:v>
+      </x:c>
+      <x:c r="O37" s="27" t="n">
+        <x:v>30091.698</x:v>
+      </x:c>
+      <x:c r="P37" s="27"/>
+      <x:c r="Q37" s="27"/>
+      <x:c r="R37" s="27"/>
+      <x:c r="S37" s="27" t="n">
+        <x:v>17210.386</x:v>
+      </x:c>
+      <x:c r="T37" s="27" t="n">
+        <x:v>15695.841</x:v>
+      </x:c>
+      <x:c r="U37" s="27" t="n">
+        <x:v>4932.278</x:v>
+      </x:c>
+      <x:c r="V37" s="27" t="n">
+        <x:v>3944.45</x:v>
+      </x:c>
+      <x:c r="W37" s="27"/>
+      <x:c r="X37" s="27"/>
+      <x:c r="Y37" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F37,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>182284.18099999998</x:v>
       </x:c>
-      <x:c r="Q37" s="27" t="n">
+      <x:c r="Z37" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F37)</x:f>
         <x:v>12</x:v>
       </x:c>
-      <x:c r="R37" s="23" t="str">
+      <x:c r="AA37" s="23" t="str">
         <x:v>缺少：Recipe - Qwen总结</x:v>
       </x:c>
     </x:row>
@@ -4368,39 +4668,46 @@
       <x:c r="G38" s="23" t="str">
         <x:v>查询5G小区CBN-福州仓山-火车南站东南美化塔C-HRHH-518和CBN-福州仓山-福厦高铁鸡笼山隧道C-HRRH-513的机械下倾角，筛选出机械下倾角在3到9之间的小区名称和机械下倾角。</x:v>
       </x:c>
-      <x:c r="H38" s="23" t="str">
-        <x:v>14994.5 ms</x:v>
-      </x:c>
-      <x:c r="I38" s="23" t="str">
-        <x:v>9674.1 ms</x:v>
-      </x:c>
-      <x:c r="J38" s="23" t="str">
-        <x:v>14894.3 ms</x:v>
-      </x:c>
-      <x:c r="K38" s="23" t="str">
-        <x:v>1662.2 ms</x:v>
-      </x:c>
-      <x:c r="L38" s="23" t="str">
-        <x:v>1998.6 ms</x:v>
-      </x:c>
-      <x:c r="M38" s="23" t="str">
-        <x:v>15177.4 ms</x:v>
-      </x:c>
-      <x:c r="N38" s="23" t="str">
-        <x:v>6244.3 ms</x:v>
-      </x:c>
-      <x:c r="O38" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H38" s="27" t="n">
+        <x:v>14994.494</x:v>
+      </x:c>
+      <x:c r="I38" s="27" t="n">
+        <x:v>9674.122</x:v>
+      </x:c>
+      <x:c r="J38" s="27" t="n">
+        <x:v>14894.279</x:v>
+      </x:c>
+      <x:c r="K38" s="27"/>
+      <x:c r="L38" s="27"/>
+      <x:c r="M38" s="27"/>
+      <x:c r="N38" s="27"/>
+      <x:c r="O38" s="27"/>
       <x:c r="P38" s="27" t="n">
+        <x:v>1662.249</x:v>
+      </x:c>
+      <x:c r="Q38" s="27"/>
+      <x:c r="R38" s="27" t="n">
+        <x:v>1998.631</x:v>
+      </x:c>
+      <x:c r="S38" s="27" t="n">
+        <x:v>15177.392</x:v>
+      </x:c>
+      <x:c r="T38" s="27" t="n">
+        <x:v>6244.334</x:v>
+      </x:c>
+      <x:c r="U38" s="27"/>
+      <x:c r="V38" s="27"/>
+      <x:c r="W38" s="27"/>
+      <x:c r="X38" s="27"/>
+      <x:c r="Y38" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F38,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>64645.50100000001</x:v>
       </x:c>
-      <x:c r="Q38" s="27" t="n">
+      <x:c r="Z38" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F38)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R38" s="23" t="str">
+      <x:c r="AA38" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4426,39 +4733,46 @@
       <x:c r="G39" s="23" t="str">
         <x:v>查询小区CBN-深圳梅沙湾U-H5H-0712的站点名称、方位角、电子下倾角，条件是方位角等于180且电子下倾角不低于6</x:v>
       </x:c>
-      <x:c r="H39" s="23" t="str">
-        <x:v>5983.4 ms</x:v>
-      </x:c>
-      <x:c r="I39" s="23" t="str">
-        <x:v>14612.2 ms</x:v>
-      </x:c>
-      <x:c r="J39" s="23" t="str">
-        <x:v>4331.3 ms</x:v>
-      </x:c>
-      <x:c r="K39" s="23" t="str">
-        <x:v>1272.9 ms</x:v>
-      </x:c>
-      <x:c r="L39" s="23" t="str">
-        <x:v>1949.8 ms</x:v>
-      </x:c>
-      <x:c r="M39" s="23" t="str">
-        <x:v>13327.6 ms</x:v>
-      </x:c>
-      <x:c r="N39" s="23" t="str">
-        <x:v>12130.2 ms</x:v>
-      </x:c>
-      <x:c r="O39" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H39" s="27" t="n">
+        <x:v>5983.37</x:v>
+      </x:c>
+      <x:c r="I39" s="27" t="n">
+        <x:v>14612.209</x:v>
+      </x:c>
+      <x:c r="J39" s="27" t="n">
+        <x:v>4331.255</x:v>
+      </x:c>
+      <x:c r="K39" s="27"/>
+      <x:c r="L39" s="27"/>
+      <x:c r="M39" s="27"/>
+      <x:c r="N39" s="27"/>
+      <x:c r="O39" s="27"/>
       <x:c r="P39" s="27" t="n">
+        <x:v>1272.895</x:v>
+      </x:c>
+      <x:c r="Q39" s="27"/>
+      <x:c r="R39" s="27" t="n">
+        <x:v>1949.797</x:v>
+      </x:c>
+      <x:c r="S39" s="27" t="n">
+        <x:v>13327.586</x:v>
+      </x:c>
+      <x:c r="T39" s="27" t="n">
+        <x:v>12130.238</x:v>
+      </x:c>
+      <x:c r="U39" s="27"/>
+      <x:c r="V39" s="27"/>
+      <x:c r="W39" s="27"/>
+      <x:c r="X39" s="27"/>
+      <x:c r="Y39" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F39,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>53607.35</x:v>
       </x:c>
-      <x:c r="Q39" s="27" t="n">
+      <x:c r="Z39" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F39)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R39" s="23" t="str">
+      <x:c r="AA39" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4484,39 +4798,46 @@
       <x:c r="G40" s="23" t="str">
         <x:v>查询深圳东海岸三D-HRH和深圳奥特莱斯D-HRH这两个站点下，NR制式中方位角为90或270的小区，返回小区名称和方位角。</x:v>
       </x:c>
-      <x:c r="H40" s="23" t="str">
-        <x:v>20043.2 ms</x:v>
-      </x:c>
-      <x:c r="I40" s="23" t="str">
-        <x:v>15059.4 ms</x:v>
-      </x:c>
-      <x:c r="J40" s="23" t="str">
-        <x:v>16443.1 ms</x:v>
-      </x:c>
-      <x:c r="K40" s="23" t="str">
-        <x:v>1631.3 ms</x:v>
-      </x:c>
-      <x:c r="L40" s="23" t="str">
-        <x:v>2503.8 ms</x:v>
-      </x:c>
-      <x:c r="M40" s="23" t="str">
-        <x:v>17309.8 ms</x:v>
-      </x:c>
-      <x:c r="N40" s="23" t="str">
-        <x:v>12226.0 ms</x:v>
-      </x:c>
-      <x:c r="O40" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H40" s="27" t="n">
+        <x:v>20043.177</x:v>
+      </x:c>
+      <x:c r="I40" s="27" t="n">
+        <x:v>15059.428</x:v>
+      </x:c>
+      <x:c r="J40" s="27" t="n">
+        <x:v>16443.072</x:v>
+      </x:c>
+      <x:c r="K40" s="27"/>
+      <x:c r="L40" s="27"/>
+      <x:c r="M40" s="27"/>
+      <x:c r="N40" s="27"/>
+      <x:c r="O40" s="27"/>
       <x:c r="P40" s="27" t="n">
+        <x:v>1631.348</x:v>
+      </x:c>
+      <x:c r="Q40" s="27"/>
+      <x:c r="R40" s="27" t="n">
+        <x:v>2503.795</x:v>
+      </x:c>
+      <x:c r="S40" s="27" t="n">
+        <x:v>17309.794</x:v>
+      </x:c>
+      <x:c r="T40" s="27" t="n">
+        <x:v>12225.98</x:v>
+      </x:c>
+      <x:c r="U40" s="27"/>
+      <x:c r="V40" s="27"/>
+      <x:c r="W40" s="27"/>
+      <x:c r="X40" s="27"/>
+      <x:c r="Y40" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F40,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>85216.594</x:v>
       </x:c>
-      <x:c r="Q40" s="27" t="n">
+      <x:c r="Z40" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F40)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R40" s="23" t="str">
+      <x:c r="AA40" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4542,39 +4863,46 @@
       <x:c r="G41" s="23" t="str">
         <x:v>查询小区 CBN-福州晋安-东浦新村4号楼C-HRHH-512 的工程参数，排除天线高度等于20米的情况，返回小区名称、天线高度和经度。</x:v>
       </x:c>
-      <x:c r="H41" s="23" t="str">
-        <x:v>8402.5 ms</x:v>
-      </x:c>
-      <x:c r="I41" s="23" t="str">
-        <x:v>17481.1 ms</x:v>
-      </x:c>
-      <x:c r="J41" s="23" t="str">
-        <x:v>19833.1 ms</x:v>
-      </x:c>
-      <x:c r="K41" s="23" t="str">
-        <x:v>1583.5 ms</x:v>
-      </x:c>
-      <x:c r="L41" s="23" t="str">
-        <x:v>2490.6 ms</x:v>
-      </x:c>
-      <x:c r="M41" s="23" t="str">
-        <x:v>30706.3 ms</x:v>
-      </x:c>
-      <x:c r="N41" s="23" t="str">
-        <x:v>16942.5 ms</x:v>
-      </x:c>
-      <x:c r="O41" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H41" s="27" t="n">
+        <x:v>8402.453</x:v>
+      </x:c>
+      <x:c r="I41" s="27" t="n">
+        <x:v>17481.125</x:v>
+      </x:c>
+      <x:c r="J41" s="27" t="n">
+        <x:v>19833.145</x:v>
+      </x:c>
+      <x:c r="K41" s="27"/>
+      <x:c r="L41" s="27"/>
+      <x:c r="M41" s="27"/>
+      <x:c r="N41" s="27"/>
+      <x:c r="O41" s="27"/>
       <x:c r="P41" s="27" t="n">
+        <x:v>1583.485</x:v>
+      </x:c>
+      <x:c r="Q41" s="27"/>
+      <x:c r="R41" s="27" t="n">
+        <x:v>2490.584</x:v>
+      </x:c>
+      <x:c r="S41" s="27" t="n">
+        <x:v>30706.304</x:v>
+      </x:c>
+      <x:c r="T41" s="27" t="n">
+        <x:v>16942.473</x:v>
+      </x:c>
+      <x:c r="U41" s="27"/>
+      <x:c r="V41" s="27"/>
+      <x:c r="W41" s="27"/>
+      <x:c r="X41" s="27"/>
+      <x:c r="Y41" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F41,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>97439.569</x:v>
       </x:c>
-      <x:c r="Q41" s="27" t="n">
+      <x:c r="Z41" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F41)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R41" s="23" t="str">
+      <x:c r="AA41" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4600,39 +4928,46 @@
       <x:c r="G42" s="23" t="str">
         <x:v>查询深圳奥特莱斯D-HRH-1小区的方位角和天线高度工程参数。</x:v>
       </x:c>
-      <x:c r="H42" s="23" t="str">
-        <x:v>14244.3 ms</x:v>
-      </x:c>
-      <x:c r="I42" s="23" t="str">
-        <x:v>18682.1 ms</x:v>
-      </x:c>
-      <x:c r="J42" s="23" t="str">
-        <x:v>10219.2 ms</x:v>
-      </x:c>
-      <x:c r="K42" s="23" t="str">
-        <x:v>1270.8 ms</x:v>
-      </x:c>
-      <x:c r="L42" s="23" t="str">
-        <x:v>1371.6 ms</x:v>
-      </x:c>
-      <x:c r="M42" s="23" t="str">
-        <x:v>2620.2 ms</x:v>
-      </x:c>
-      <x:c r="N42" s="23" t="str">
-        <x:v>3527.5 ms</x:v>
-      </x:c>
-      <x:c r="O42" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H42" s="27" t="n">
+        <x:v>14244.333</x:v>
+      </x:c>
+      <x:c r="I42" s="27" t="n">
+        <x:v>18682.083</x:v>
+      </x:c>
+      <x:c r="J42" s="27" t="n">
+        <x:v>10219.216</x:v>
+      </x:c>
+      <x:c r="K42" s="27"/>
+      <x:c r="L42" s="27"/>
+      <x:c r="M42" s="27"/>
+      <x:c r="N42" s="27"/>
+      <x:c r="O42" s="27"/>
       <x:c r="P42" s="27" t="n">
+        <x:v>1270.835</x:v>
+      </x:c>
+      <x:c r="Q42" s="27"/>
+      <x:c r="R42" s="27" t="n">
+        <x:v>1371.565</x:v>
+      </x:c>
+      <x:c r="S42" s="27" t="n">
+        <x:v>2620.244</x:v>
+      </x:c>
+      <x:c r="T42" s="27" t="n">
+        <x:v>3527.501</x:v>
+      </x:c>
+      <x:c r="U42" s="27"/>
+      <x:c r="V42" s="27"/>
+      <x:c r="W42" s="27"/>
+      <x:c r="X42" s="27"/>
+      <x:c r="Y42" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F42,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>51935.777</x:v>
       </x:c>
-      <x:c r="Q42" s="27" t="n">
+      <x:c r="Z42" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F42)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R42" s="23" t="str">
+      <x:c r="AA42" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4658,39 +4993,46 @@
       <x:c r="G43" s="23" t="str">
         <x:v>查询CBN-深圳梅沙湾二U-H5H站点下的小区名称和经度</x:v>
       </x:c>
-      <x:c r="H43" s="23" t="str">
-        <x:v>3435.8 ms</x:v>
-      </x:c>
-      <x:c r="I43" s="23" t="str">
-        <x:v>3159.8 ms</x:v>
-      </x:c>
-      <x:c r="J43" s="23" t="str">
-        <x:v>2352.6 ms</x:v>
-      </x:c>
-      <x:c r="K43" s="23" t="str">
-        <x:v>1311.1 ms</x:v>
-      </x:c>
-      <x:c r="L43" s="23" t="str">
-        <x:v>2488.2 ms</x:v>
-      </x:c>
-      <x:c r="M43" s="23" t="str">
-        <x:v>4712.2 ms</x:v>
-      </x:c>
-      <x:c r="N43" s="23" t="str">
-        <x:v>4166.3 ms</x:v>
-      </x:c>
-      <x:c r="O43" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H43" s="27" t="n">
+        <x:v>3435.841</x:v>
+      </x:c>
+      <x:c r="I43" s="27" t="n">
+        <x:v>3159.773</x:v>
+      </x:c>
+      <x:c r="J43" s="27" t="n">
+        <x:v>2352.61</x:v>
+      </x:c>
+      <x:c r="K43" s="27"/>
+      <x:c r="L43" s="27"/>
+      <x:c r="M43" s="27"/>
+      <x:c r="N43" s="27"/>
+      <x:c r="O43" s="27"/>
       <x:c r="P43" s="27" t="n">
+        <x:v>1311.051</x:v>
+      </x:c>
+      <x:c r="Q43" s="27"/>
+      <x:c r="R43" s="27" t="n">
+        <x:v>2488.213</x:v>
+      </x:c>
+      <x:c r="S43" s="27" t="n">
+        <x:v>4712.228</x:v>
+      </x:c>
+      <x:c r="T43" s="27" t="n">
+        <x:v>4166.295</x:v>
+      </x:c>
+      <x:c r="U43" s="27"/>
+      <x:c r="V43" s="27"/>
+      <x:c r="W43" s="27"/>
+      <x:c r="X43" s="27"/>
+      <x:c r="Y43" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F43,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>21626.011</x:v>
       </x:c>
-      <x:c r="Q43" s="27" t="n">
+      <x:c r="Z43" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F43)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R43" s="23" t="str">
+      <x:c r="AA43" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4716,39 +5058,46 @@
       <x:c r="G44" s="23" t="str">
         <x:v>查询小区 CBN-福州晋安-东浦新村4号楼C-HRHH-513 的电子下倾角和基站标识是多少</x:v>
       </x:c>
-      <x:c r="H44" s="23" t="str">
-        <x:v>3454.4 ms</x:v>
-      </x:c>
-      <x:c r="I44" s="23" t="str">
-        <x:v>3489.1 ms</x:v>
-      </x:c>
-      <x:c r="J44" s="23" t="str">
-        <x:v>2471.6 ms</x:v>
-      </x:c>
-      <x:c r="K44" s="23" t="str">
-        <x:v>1272.5 ms</x:v>
-      </x:c>
-      <x:c r="L44" s="23" t="str">
-        <x:v>1438.6 ms</x:v>
-      </x:c>
-      <x:c r="M44" s="23" t="str">
-        <x:v>2411.2 ms</x:v>
-      </x:c>
-      <x:c r="N44" s="23" t="str">
-        <x:v>3476.4 ms</x:v>
-      </x:c>
-      <x:c r="O44" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H44" s="27" t="n">
+        <x:v>3454.4</x:v>
+      </x:c>
+      <x:c r="I44" s="27" t="n">
+        <x:v>3489.123</x:v>
+      </x:c>
+      <x:c r="J44" s="27" t="n">
+        <x:v>2471.581</x:v>
+      </x:c>
+      <x:c r="K44" s="27"/>
+      <x:c r="L44" s="27"/>
+      <x:c r="M44" s="27"/>
+      <x:c r="N44" s="27"/>
+      <x:c r="O44" s="27"/>
       <x:c r="P44" s="27" t="n">
+        <x:v>1272.45</x:v>
+      </x:c>
+      <x:c r="Q44" s="27"/>
+      <x:c r="R44" s="27" t="n">
+        <x:v>1438.58</x:v>
+      </x:c>
+      <x:c r="S44" s="27" t="n">
+        <x:v>2411.229</x:v>
+      </x:c>
+      <x:c r="T44" s="27" t="n">
+        <x:v>3476.405</x:v>
+      </x:c>
+      <x:c r="U44" s="27"/>
+      <x:c r="V44" s="27"/>
+      <x:c r="W44" s="27"/>
+      <x:c r="X44" s="27"/>
+      <x:c r="Y44" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F44,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18013.768</x:v>
       </x:c>
-      <x:c r="Q44" s="27" t="n">
+      <x:c r="Z44" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F44)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R44" s="23" t="str">
+      <x:c r="AA44" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4774,39 +5123,46 @@
       <x:c r="G45" s="23" t="str">
         <x:v>查询深圳大梅沙D-HRH-1小区的CGI和站点名称</x:v>
       </x:c>
-      <x:c r="H45" s="23" t="str">
-        <x:v>2758.8 ms</x:v>
-      </x:c>
-      <x:c r="I45" s="23" t="str">
-        <x:v>3063.8 ms</x:v>
-      </x:c>
-      <x:c r="J45" s="23" t="str">
-        <x:v>1800.2 ms</x:v>
-      </x:c>
-      <x:c r="K45" s="23" t="str">
-        <x:v>1234.1 ms</x:v>
-      </x:c>
-      <x:c r="L45" s="23" t="str">
-        <x:v>1479.8 ms</x:v>
-      </x:c>
-      <x:c r="M45" s="23" t="str">
-        <x:v>2385.0 ms</x:v>
-      </x:c>
-      <x:c r="N45" s="23" t="str">
-        <x:v>3977.1 ms</x:v>
-      </x:c>
-      <x:c r="O45" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H45" s="27" t="n">
+        <x:v>2758.794</x:v>
+      </x:c>
+      <x:c r="I45" s="27" t="n">
+        <x:v>3063.82</x:v>
+      </x:c>
+      <x:c r="J45" s="27" t="n">
+        <x:v>1800.248</x:v>
+      </x:c>
+      <x:c r="K45" s="27"/>
+      <x:c r="L45" s="27"/>
+      <x:c r="M45" s="27"/>
+      <x:c r="N45" s="27"/>
+      <x:c r="O45" s="27"/>
       <x:c r="P45" s="27" t="n">
+        <x:v>1234.132</x:v>
+      </x:c>
+      <x:c r="Q45" s="27"/>
+      <x:c r="R45" s="27" t="n">
+        <x:v>1479.827</x:v>
+      </x:c>
+      <x:c r="S45" s="27" t="n">
+        <x:v>2385.032</x:v>
+      </x:c>
+      <x:c r="T45" s="27" t="n">
+        <x:v>3977.11</x:v>
+      </x:c>
+      <x:c r="U45" s="27"/>
+      <x:c r="V45" s="27"/>
+      <x:c r="W45" s="27"/>
+      <x:c r="X45" s="27"/>
+      <x:c r="Y45" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F45,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>16698.963</x:v>
       </x:c>
-      <x:c r="Q45" s="27" t="n">
+      <x:c r="Z45" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F45)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R45" s="23" t="str">
+      <x:c r="AA45" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4832,39 +5188,46 @@
       <x:c r="G46" s="23" t="str">
         <x:v>查询深圳东华风车D-HRH站点下小区的方位角和移动网号</x:v>
       </x:c>
-      <x:c r="H46" s="23" t="str">
-        <x:v>3606.8 ms</x:v>
-      </x:c>
-      <x:c r="I46" s="23" t="str">
-        <x:v>3328.3 ms</x:v>
-      </x:c>
-      <x:c r="J46" s="23" t="str">
-        <x:v>2240.0 ms</x:v>
-      </x:c>
-      <x:c r="K46" s="23" t="str">
-        <x:v>1213.7 ms</x:v>
-      </x:c>
-      <x:c r="L46" s="23" t="str">
-        <x:v>1565.3 ms</x:v>
-      </x:c>
-      <x:c r="M46" s="23" t="str">
-        <x:v>3034.4 ms</x:v>
-      </x:c>
-      <x:c r="N46" s="23" t="str">
-        <x:v>3144.3 ms</x:v>
-      </x:c>
-      <x:c r="O46" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H46" s="27" t="n">
+        <x:v>3606.819</x:v>
+      </x:c>
+      <x:c r="I46" s="27" t="n">
+        <x:v>3328.343</x:v>
+      </x:c>
+      <x:c r="J46" s="27" t="n">
+        <x:v>2239.97</x:v>
+      </x:c>
+      <x:c r="K46" s="27"/>
+      <x:c r="L46" s="27"/>
+      <x:c r="M46" s="27"/>
+      <x:c r="N46" s="27"/>
+      <x:c r="O46" s="27"/>
       <x:c r="P46" s="27" t="n">
+        <x:v>1213.723</x:v>
+      </x:c>
+      <x:c r="Q46" s="27"/>
+      <x:c r="R46" s="27" t="n">
+        <x:v>1565.263</x:v>
+      </x:c>
+      <x:c r="S46" s="27" t="n">
+        <x:v>3034.37</x:v>
+      </x:c>
+      <x:c r="T46" s="27" t="n">
+        <x:v>3144.254</x:v>
+      </x:c>
+      <x:c r="U46" s="27"/>
+      <x:c r="V46" s="27"/>
+      <x:c r="W46" s="27"/>
+      <x:c r="X46" s="27"/>
+      <x:c r="Y46" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F46,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18132.742</x:v>
       </x:c>
-      <x:c r="Q46" s="27" t="n">
+      <x:c r="Z46" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F46)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R46" s="23" t="str">
+      <x:c r="AA46" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4890,39 +5253,48 @@
       <x:c r="G47" s="23" t="str">
         <x:v>查询深圳梅沙湾D-HRH-3和深圳梅沙湾二D-HRH-1这两个小区的方位角、电子下倾角以及设备厂商。</x:v>
       </x:c>
-      <x:c r="H47" s="23" t="str">
-        <x:v>3241.8 ms</x:v>
-      </x:c>
-      <x:c r="I47" s="23" t="str">
-        <x:v>3127.7 ms</x:v>
-      </x:c>
-      <x:c r="J47" s="23" t="str">
-        <x:v>2456.2 ms</x:v>
-      </x:c>
-      <x:c r="K47" s="23" t="str">
-        <x:v>第1次 1302.3 ms；第2次 1656.0 ms</x:v>
-      </x:c>
-      <x:c r="L47" s="23" t="str">
-        <x:v>2320.6 ms</x:v>
-      </x:c>
-      <x:c r="M47" s="23" t="str">
-        <x:v>3195.3 ms</x:v>
-      </x:c>
-      <x:c r="N47" s="23" t="str">
-        <x:v>2886.1 ms</x:v>
-      </x:c>
-      <x:c r="O47" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H47" s="27" t="n">
+        <x:v>3241.838</x:v>
+      </x:c>
+      <x:c r="I47" s="27" t="n">
+        <x:v>3127.676</x:v>
+      </x:c>
+      <x:c r="J47" s="27" t="n">
+        <x:v>2456.22</x:v>
+      </x:c>
+      <x:c r="K47" s="27"/>
+      <x:c r="L47" s="27"/>
+      <x:c r="M47" s="27"/>
+      <x:c r="N47" s="27"/>
+      <x:c r="O47" s="27"/>
       <x:c r="P47" s="27" t="n">
+        <x:v>1302.324</x:v>
+      </x:c>
+      <x:c r="Q47" s="27" t="n">
+        <x:v>1656.016</x:v>
+      </x:c>
+      <x:c r="R47" s="27" t="n">
+        <x:v>2320.568</x:v>
+      </x:c>
+      <x:c r="S47" s="27" t="n">
+        <x:v>3195.307</x:v>
+      </x:c>
+      <x:c r="T47" s="27" t="n">
+        <x:v>2886.139</x:v>
+      </x:c>
+      <x:c r="U47" s="27"/>
+      <x:c r="V47" s="27"/>
+      <x:c r="W47" s="27"/>
+      <x:c r="X47" s="27"/>
+      <x:c r="Y47" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F47,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>20186.088</x:v>
       </x:c>
-      <x:c r="Q47" s="27" t="n">
+      <x:c r="Z47" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F47)</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="R47" s="23" t="str">
+      <x:c r="AA47" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -4948,39 +5320,46 @@
       <x:c r="G48" s="23" t="str">
         <x:v>查询CBN-深圳大梅沙U-H5H和深圳大梅沙二D-HRH这两个站点下小区的纬度、机械下倾角和小区标识</x:v>
       </x:c>
-      <x:c r="H48" s="23" t="str">
-        <x:v>4456.8 ms</x:v>
-      </x:c>
-      <x:c r="I48" s="23" t="str">
-        <x:v>3618.6 ms</x:v>
-      </x:c>
-      <x:c r="J48" s="23" t="str">
-        <x:v>2760.2 ms</x:v>
-      </x:c>
-      <x:c r="K48" s="23" t="str">
-        <x:v>1403.0 ms</x:v>
-      </x:c>
-      <x:c r="L48" s="23" t="str">
-        <x:v>3121.2 ms</x:v>
-      </x:c>
-      <x:c r="M48" s="23" t="str">
-        <x:v>6332.0 ms</x:v>
-      </x:c>
-      <x:c r="N48" s="23" t="str">
-        <x:v>3425.0 ms</x:v>
-      </x:c>
-      <x:c r="O48" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H48" s="27" t="n">
+        <x:v>4456.84</x:v>
+      </x:c>
+      <x:c r="I48" s="27" t="n">
+        <x:v>3618.556</x:v>
+      </x:c>
+      <x:c r="J48" s="27" t="n">
+        <x:v>2760.245</x:v>
+      </x:c>
+      <x:c r="K48" s="27"/>
+      <x:c r="L48" s="27"/>
+      <x:c r="M48" s="27"/>
+      <x:c r="N48" s="27"/>
+      <x:c r="O48" s="27"/>
       <x:c r="P48" s="27" t="n">
+        <x:v>1403.042</x:v>
+      </x:c>
+      <x:c r="Q48" s="27"/>
+      <x:c r="R48" s="27" t="n">
+        <x:v>3121.214</x:v>
+      </x:c>
+      <x:c r="S48" s="27" t="n">
+        <x:v>6332.047</x:v>
+      </x:c>
+      <x:c r="T48" s="27" t="n">
+        <x:v>3425.032</x:v>
+      </x:c>
+      <x:c r="U48" s="27"/>
+      <x:c r="V48" s="27"/>
+      <x:c r="W48" s="27"/>
+      <x:c r="X48" s="27"/>
+      <x:c r="Y48" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F48,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>25116.976</x:v>
       </x:c>
-      <x:c r="Q48" s="27" t="n">
+      <x:c r="Z48" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F48)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R48" s="23" t="str">
+      <x:c r="AA48" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5006,39 +5385,52 @@
       <x:c r="G49" s="23" t="str">
         <x:v>查询小区 CBN-福州仓山-福厦高铁鸡笼山隧道C-HRRH-513、CBN-福州仓山-火车南站东南美化塔C-HRHH-518、CBN-福州仓山-永南路与站后路交叉口C-HRHH-516 这三个小区的基站标识、移动网号和天线高度，并进行对比。</x:v>
       </x:c>
-      <x:c r="H49" s="23" t="str">
-        <x:v>3631.3 ms</x:v>
-      </x:c>
-      <x:c r="I49" s="23" t="str">
-        <x:v>3216.7 ms</x:v>
-      </x:c>
-      <x:c r="J49" s="23" t="str">
-        <x:v>2691.9 ms</x:v>
-      </x:c>
-      <x:c r="K49" s="23" t="str">
-        <x:v>1902.2 ms</x:v>
-      </x:c>
-      <x:c r="L49" s="23" t="str">
-        <x:v>3098.1 ms</x:v>
-      </x:c>
-      <x:c r="M49" s="23" t="str">
-        <x:v>4899.1 ms</x:v>
-      </x:c>
-      <x:c r="N49" s="23" t="str">
-        <x:v>4139.5 ms</x:v>
-      </x:c>
-      <x:c r="O49" s="23" t="str">
-        <x:v>第1次 ToolSearch: 2494.2 ms；第2次 ToolSearch: 2126.5 ms；第3次 Glob: 2574.3 ms</x:v>
-      </x:c>
+      <x:c r="H49" s="27" t="n">
+        <x:v>3631.259</x:v>
+      </x:c>
+      <x:c r="I49" s="27" t="n">
+        <x:v>3216.722</x:v>
+      </x:c>
+      <x:c r="J49" s="27" t="n">
+        <x:v>2691.861</x:v>
+      </x:c>
+      <x:c r="K49" s="27"/>
+      <x:c r="L49" s="27"/>
+      <x:c r="M49" s="27"/>
+      <x:c r="N49" s="27"/>
+      <x:c r="O49" s="27"/>
       <x:c r="P49" s="27" t="n">
+        <x:v>1902.207</x:v>
+      </x:c>
+      <x:c r="Q49" s="27"/>
+      <x:c r="R49" s="27" t="n">
+        <x:v>3098.128</x:v>
+      </x:c>
+      <x:c r="S49" s="27" t="n">
+        <x:v>4899.083</x:v>
+      </x:c>
+      <x:c r="T49" s="27" t="n">
+        <x:v>4139.455</x:v>
+      </x:c>
+      <x:c r="U49" s="27" t="n">
+        <x:v>2494.187</x:v>
+      </x:c>
+      <x:c r="V49" s="27" t="n">
+        <x:v>2126.464</x:v>
+      </x:c>
+      <x:c r="W49" s="27" t="n">
+        <x:v>2574.269</x:v>
+      </x:c>
+      <x:c r="X49" s="27"/>
+      <x:c r="Y49" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F49,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>30773.635000000002</x:v>
       </x:c>
-      <x:c r="Q49" s="27" t="n">
+      <x:c r="Z49" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F49)</x:f>
         <x:v>10</x:v>
       </x:c>
-      <x:c r="R49" s="23" t="str">
+      <x:c r="AA49" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5064,39 +5456,46 @@
       <x:c r="G50" s="23" t="str">
         <x:v>查询深圳东海岸三D-HRH-1小区和深圳奥特莱斯D-HRH-3小区的经度和站点名称。</x:v>
       </x:c>
-      <x:c r="H50" s="23" t="str">
-        <x:v>3219.8 ms</x:v>
-      </x:c>
-      <x:c r="I50" s="23" t="str">
-        <x:v>2723.8 ms</x:v>
-      </x:c>
-      <x:c r="J50" s="23" t="str">
-        <x:v>1656.4 ms</x:v>
-      </x:c>
-      <x:c r="K50" s="23" t="str">
-        <x:v>1282.7 ms</x:v>
-      </x:c>
-      <x:c r="L50" s="23" t="str">
-        <x:v>1612.8 ms</x:v>
-      </x:c>
-      <x:c r="M50" s="23" t="str">
-        <x:v>2232.9 ms</x:v>
-      </x:c>
-      <x:c r="N50" s="23" t="str">
-        <x:v>3544.0 ms</x:v>
-      </x:c>
-      <x:c r="O50" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H50" s="27" t="n">
+        <x:v>3219.775</x:v>
+      </x:c>
+      <x:c r="I50" s="27" t="n">
+        <x:v>2723.771</x:v>
+      </x:c>
+      <x:c r="J50" s="27" t="n">
+        <x:v>1656.44</x:v>
+      </x:c>
+      <x:c r="K50" s="27"/>
+      <x:c r="L50" s="27"/>
+      <x:c r="M50" s="27"/>
+      <x:c r="N50" s="27"/>
+      <x:c r="O50" s="27"/>
       <x:c r="P50" s="27" t="n">
+        <x:v>1282.708</x:v>
+      </x:c>
+      <x:c r="Q50" s="27"/>
+      <x:c r="R50" s="27" t="n">
+        <x:v>1612.813</x:v>
+      </x:c>
+      <x:c r="S50" s="27" t="n">
+        <x:v>2232.878</x:v>
+      </x:c>
+      <x:c r="T50" s="27" t="n">
+        <x:v>3544.049</x:v>
+      </x:c>
+      <x:c r="U50" s="27"/>
+      <x:c r="V50" s="27"/>
+      <x:c r="W50" s="27"/>
+      <x:c r="X50" s="27"/>
+      <x:c r="Y50" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F50,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>16272.434000000001</x:v>
       </x:c>
-      <x:c r="Q50" s="27" t="n">
+      <x:c r="Z50" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F50)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R50" s="23" t="str">
+      <x:c r="AA50" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5122,39 +5521,46 @@
       <x:c r="G51" s="23" t="str">
         <x:v>查询站点CBN-福州马尾-高铁鼓山1号隧道出口（左侧）C-HRRH和CBN-深圳东华风车U-H5H下所有小区的方位角、电子下倾角和机械下倾角</x:v>
       </x:c>
-      <x:c r="H51" s="23" t="str">
-        <x:v>3589.0 ms</x:v>
-      </x:c>
-      <x:c r="I51" s="23" t="str">
-        <x:v>2955.8 ms</x:v>
-      </x:c>
-      <x:c r="J51" s="23" t="str">
-        <x:v>1990.2 ms</x:v>
-      </x:c>
-      <x:c r="K51" s="23" t="str">
-        <x:v>1399.4 ms</x:v>
-      </x:c>
-      <x:c r="L51" s="23" t="str">
-        <x:v>2774.1 ms</x:v>
-      </x:c>
-      <x:c r="M51" s="23" t="str">
-        <x:v>3917.2 ms</x:v>
-      </x:c>
-      <x:c r="N51" s="23" t="str">
-        <x:v>3953.5 ms</x:v>
-      </x:c>
-      <x:c r="O51" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H51" s="27" t="n">
+        <x:v>3588.974</x:v>
+      </x:c>
+      <x:c r="I51" s="27" t="n">
+        <x:v>2955.785</x:v>
+      </x:c>
+      <x:c r="J51" s="27" t="n">
+        <x:v>1990.221</x:v>
+      </x:c>
+      <x:c r="K51" s="27"/>
+      <x:c r="L51" s="27"/>
+      <x:c r="M51" s="27"/>
+      <x:c r="N51" s="27"/>
+      <x:c r="O51" s="27"/>
       <x:c r="P51" s="27" t="n">
+        <x:v>1399.359</x:v>
+      </x:c>
+      <x:c r="Q51" s="27"/>
+      <x:c r="R51" s="27" t="n">
+        <x:v>2774.146</x:v>
+      </x:c>
+      <x:c r="S51" s="27" t="n">
+        <x:v>3917.182</x:v>
+      </x:c>
+      <x:c r="T51" s="27" t="n">
+        <x:v>3953.534</x:v>
+      </x:c>
+      <x:c r="U51" s="27"/>
+      <x:c r="V51" s="27"/>
+      <x:c r="W51" s="27"/>
+      <x:c r="X51" s="27"/>
+      <x:c r="Y51" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F51,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>20579.201</x:v>
       </x:c>
-      <x:c r="Q51" s="27" t="n">
+      <x:c r="Z51" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F51)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R51" s="23" t="str">
+      <x:c r="AA51" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5180,39 +5586,46 @@
       <x:c r="G52" s="23" t="str">
         <x:v>查询深圳大梅沙D-HRH站点下5G小区的方位角和电子下倾角工程参数</x:v>
       </x:c>
-      <x:c r="H52" s="23" t="str">
-        <x:v>3531.6 ms</x:v>
-      </x:c>
-      <x:c r="I52" s="23" t="str">
-        <x:v>2959.1 ms</x:v>
-      </x:c>
-      <x:c r="J52" s="23" t="str">
-        <x:v>1622.6 ms</x:v>
-      </x:c>
-      <x:c r="K52" s="23" t="str">
-        <x:v>1314.6 ms</x:v>
-      </x:c>
-      <x:c r="L52" s="23" t="str">
-        <x:v>2174.0 ms</x:v>
-      </x:c>
-      <x:c r="M52" s="23" t="str">
-        <x:v>3367.7 ms</x:v>
-      </x:c>
-      <x:c r="N52" s="23" t="str">
-        <x:v>3771.1 ms</x:v>
-      </x:c>
-      <x:c r="O52" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H52" s="27" t="n">
+        <x:v>3531.61</x:v>
+      </x:c>
+      <x:c r="I52" s="27" t="n">
+        <x:v>2959.135</x:v>
+      </x:c>
+      <x:c r="J52" s="27" t="n">
+        <x:v>1622.609</x:v>
+      </x:c>
+      <x:c r="K52" s="27"/>
+      <x:c r="L52" s="27"/>
+      <x:c r="M52" s="27"/>
+      <x:c r="N52" s="27"/>
+      <x:c r="O52" s="27"/>
       <x:c r="P52" s="27" t="n">
+        <x:v>1314.633</x:v>
+      </x:c>
+      <x:c r="Q52" s="27"/>
+      <x:c r="R52" s="27" t="n">
+        <x:v>2173.973</x:v>
+      </x:c>
+      <x:c r="S52" s="27" t="n">
+        <x:v>3367.682</x:v>
+      </x:c>
+      <x:c r="T52" s="27" t="n">
+        <x:v>3771.076</x:v>
+      </x:c>
+      <x:c r="U52" s="27"/>
+      <x:c r="V52" s="27"/>
+      <x:c r="W52" s="27"/>
+      <x:c r="X52" s="27"/>
+      <x:c r="Y52" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F52,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18740.718</x:v>
       </x:c>
-      <x:c r="Q52" s="27" t="n">
+      <x:c r="Z52" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F52)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R52" s="23" t="str">
+      <x:c r="AA52" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5238,39 +5651,46 @@
       <x:c r="G53" s="23" t="str">
         <x:v>查询CBN-深圳梅沙湾U-H5H-0711这个NR小区的站点名称和纬度。</x:v>
       </x:c>
-      <x:c r="H53" s="23" t="str">
-        <x:v>2701.3 ms</x:v>
-      </x:c>
-      <x:c r="I53" s="23" t="str">
-        <x:v>2704.1 ms</x:v>
-      </x:c>
-      <x:c r="J53" s="23" t="str">
-        <x:v>1559.1 ms</x:v>
-      </x:c>
-      <x:c r="K53" s="23" t="str">
-        <x:v>1454.7 ms</x:v>
-      </x:c>
-      <x:c r="L53" s="23" t="str">
-        <x:v>1427.1 ms</x:v>
-      </x:c>
-      <x:c r="M53" s="23" t="str">
-        <x:v>2102.9 ms</x:v>
-      </x:c>
-      <x:c r="N53" s="23" t="str">
-        <x:v>2873.7 ms</x:v>
-      </x:c>
-      <x:c r="O53" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H53" s="27" t="n">
+        <x:v>2701.256</x:v>
+      </x:c>
+      <x:c r="I53" s="27" t="n">
+        <x:v>2704.142</x:v>
+      </x:c>
+      <x:c r="J53" s="27" t="n">
+        <x:v>1559.133</x:v>
+      </x:c>
+      <x:c r="K53" s="27"/>
+      <x:c r="L53" s="27"/>
+      <x:c r="M53" s="27"/>
+      <x:c r="N53" s="27"/>
+      <x:c r="O53" s="27"/>
       <x:c r="P53" s="27" t="n">
+        <x:v>1454.711</x:v>
+      </x:c>
+      <x:c r="Q53" s="27"/>
+      <x:c r="R53" s="27" t="n">
+        <x:v>1427.054</x:v>
+      </x:c>
+      <x:c r="S53" s="27" t="n">
+        <x:v>2102.925</x:v>
+      </x:c>
+      <x:c r="T53" s="27" t="n">
+        <x:v>2873.724</x:v>
+      </x:c>
+      <x:c r="U53" s="27"/>
+      <x:c r="V53" s="27"/>
+      <x:c r="W53" s="27"/>
+      <x:c r="X53" s="27"/>
+      <x:c r="Y53" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F53,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>14822.944999999998</x:v>
       </x:c>
-      <x:c r="Q53" s="27" t="n">
+      <x:c r="Z53" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F53)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R53" s="23" t="str">
+      <x:c r="AA53" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5296,39 +5716,48 @@
       <x:c r="G54" s="23" t="str">
         <x:v>查询深圳奥特莱斯D-HRH-1和深圳奥特莱斯D-HRH-2这两个5G小区的经度和设备厂商。</x:v>
       </x:c>
-      <x:c r="H54" s="23" t="str">
-        <x:v>2816.9 ms</x:v>
-      </x:c>
-      <x:c r="I54" s="23" t="str">
-        <x:v>2616.1 ms</x:v>
-      </x:c>
-      <x:c r="J54" s="23" t="str">
-        <x:v>1663.3 ms</x:v>
-      </x:c>
-      <x:c r="K54" s="23" t="str">
-        <x:v>第1次 1371.4 ms；第2次 1711.8 ms</x:v>
-      </x:c>
-      <x:c r="L54" s="23" t="str">
-        <x:v>1889.9 ms</x:v>
-      </x:c>
-      <x:c r="M54" s="23" t="str">
-        <x:v>2325.7 ms</x:v>
-      </x:c>
-      <x:c r="N54" s="23" t="str">
-        <x:v>3499.7 ms</x:v>
-      </x:c>
-      <x:c r="O54" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H54" s="27" t="n">
+        <x:v>2816.923</x:v>
+      </x:c>
+      <x:c r="I54" s="27" t="n">
+        <x:v>2616.137</x:v>
+      </x:c>
+      <x:c r="J54" s="27" t="n">
+        <x:v>1663.306</x:v>
+      </x:c>
+      <x:c r="K54" s="27"/>
+      <x:c r="L54" s="27"/>
+      <x:c r="M54" s="27"/>
+      <x:c r="N54" s="27"/>
+      <x:c r="O54" s="27"/>
       <x:c r="P54" s="27" t="n">
+        <x:v>1371.379</x:v>
+      </x:c>
+      <x:c r="Q54" s="27" t="n">
+        <x:v>1711.81</x:v>
+      </x:c>
+      <x:c r="R54" s="27" t="n">
+        <x:v>1889.898</x:v>
+      </x:c>
+      <x:c r="S54" s="27" t="n">
+        <x:v>2325.74</x:v>
+      </x:c>
+      <x:c r="T54" s="27" t="n">
+        <x:v>3499.738</x:v>
+      </x:c>
+      <x:c r="U54" s="27"/>
+      <x:c r="V54" s="27"/>
+      <x:c r="W54" s="27"/>
+      <x:c r="X54" s="27"/>
+      <x:c r="Y54" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F54,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>17894.930999999997</x:v>
       </x:c>
-      <x:c r="Q54" s="27" t="n">
+      <x:c r="Z54" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F54)</x:f>
         <x:v>8</x:v>
       </x:c>
-      <x:c r="R54" s="23" t="str">
+      <x:c r="AA54" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5354,39 +5783,46 @@
       <x:c r="G55" s="23" t="str">
         <x:v>查询CBN-福州仓山-福州南站火车南站西北美化塔C-HRRH站点下NR小区的移动国家码和小区名称。</x:v>
       </x:c>
-      <x:c r="H55" s="23" t="str">
-        <x:v>3235.9 ms</x:v>
-      </x:c>
-      <x:c r="I55" s="23" t="str">
-        <x:v>2717.6 ms</x:v>
-      </x:c>
-      <x:c r="J55" s="23" t="str">
-        <x:v>1766.6 ms</x:v>
-      </x:c>
-      <x:c r="K55" s="23" t="str">
-        <x:v>1379.8 ms</x:v>
-      </x:c>
-      <x:c r="L55" s="23" t="str">
-        <x:v>1745.3 ms</x:v>
-      </x:c>
-      <x:c r="M55" s="23" t="str">
-        <x:v>2361.0 ms</x:v>
-      </x:c>
-      <x:c r="N55" s="23" t="str">
-        <x:v>3164.9 ms</x:v>
-      </x:c>
-      <x:c r="O55" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H55" s="27" t="n">
+        <x:v>3235.864</x:v>
+      </x:c>
+      <x:c r="I55" s="27" t="n">
+        <x:v>2717.586</x:v>
+      </x:c>
+      <x:c r="J55" s="27" t="n">
+        <x:v>1766.631</x:v>
+      </x:c>
+      <x:c r="K55" s="27"/>
+      <x:c r="L55" s="27"/>
+      <x:c r="M55" s="27"/>
+      <x:c r="N55" s="27"/>
+      <x:c r="O55" s="27"/>
       <x:c r="P55" s="27" t="n">
+        <x:v>1379.826</x:v>
+      </x:c>
+      <x:c r="Q55" s="27"/>
+      <x:c r="R55" s="27" t="n">
+        <x:v>1745.267</x:v>
+      </x:c>
+      <x:c r="S55" s="27" t="n">
+        <x:v>2360.973</x:v>
+      </x:c>
+      <x:c r="T55" s="27" t="n">
+        <x:v>3164.856</x:v>
+      </x:c>
+      <x:c r="U55" s="27"/>
+      <x:c r="V55" s="27"/>
+      <x:c r="W55" s="27"/>
+      <x:c r="X55" s="27"/>
+      <x:c r="Y55" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F55,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>16371.002999999999</x:v>
       </x:c>
-      <x:c r="Q55" s="27" t="n">
+      <x:c r="Z55" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F55)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R55" s="23" t="str">
+      <x:c r="AA55" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5412,39 +5848,46 @@
       <x:c r="G56" s="23" t="str">
         <x:v>查询深圳东海岸三D-HRH-1这个5G小区的方位角、电子下倾角和站点名称</x:v>
       </x:c>
-      <x:c r="H56" s="23" t="str">
-        <x:v>3007.5 ms</x:v>
-      </x:c>
-      <x:c r="I56" s="23" t="str">
-        <x:v>2714.3 ms</x:v>
-      </x:c>
-      <x:c r="J56" s="23" t="str">
-        <x:v>1555.0 ms</x:v>
-      </x:c>
-      <x:c r="K56" s="23" t="str">
-        <x:v>1356.3 ms</x:v>
-      </x:c>
-      <x:c r="L56" s="23" t="str">
-        <x:v>1466.9 ms</x:v>
-      </x:c>
-      <x:c r="M56" s="23" t="str">
-        <x:v>2434.8 ms</x:v>
-      </x:c>
-      <x:c r="N56" s="23" t="str">
-        <x:v>3417.7 ms</x:v>
-      </x:c>
-      <x:c r="O56" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H56" s="27" t="n">
+        <x:v>3007.475</x:v>
+      </x:c>
+      <x:c r="I56" s="27" t="n">
+        <x:v>2714.343</x:v>
+      </x:c>
+      <x:c r="J56" s="27" t="n">
+        <x:v>1554.951</x:v>
+      </x:c>
+      <x:c r="K56" s="27"/>
+      <x:c r="L56" s="27"/>
+      <x:c r="M56" s="27"/>
+      <x:c r="N56" s="27"/>
+      <x:c r="O56" s="27"/>
       <x:c r="P56" s="27" t="n">
+        <x:v>1356.262</x:v>
+      </x:c>
+      <x:c r="Q56" s="27"/>
+      <x:c r="R56" s="27" t="n">
+        <x:v>1466.931</x:v>
+      </x:c>
+      <x:c r="S56" s="27" t="n">
+        <x:v>2434.818</x:v>
+      </x:c>
+      <x:c r="T56" s="27" t="n">
+        <x:v>3417.716</x:v>
+      </x:c>
+      <x:c r="U56" s="27"/>
+      <x:c r="V56" s="27"/>
+      <x:c r="W56" s="27"/>
+      <x:c r="X56" s="27"/>
+      <x:c r="Y56" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F56,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>15952.496</x:v>
       </x:c>
-      <x:c r="Q56" s="27" t="n">
+      <x:c r="Z56" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F56)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R56" s="23" t="str">
+      <x:c r="AA56" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5470,39 +5913,46 @@
       <x:c r="G57" s="23" t="str">
         <x:v>查询深圳大梅沙D-HRH站点下天线高度大于30米的小区，返回小区名称、天线高度和方位角</x:v>
       </x:c>
-      <x:c r="H57" s="23" t="str">
-        <x:v>3009.8 ms</x:v>
-      </x:c>
-      <x:c r="I57" s="23" t="str">
-        <x:v>2623.6 ms</x:v>
-      </x:c>
-      <x:c r="J57" s="23" t="str">
-        <x:v>1889.8 ms</x:v>
-      </x:c>
-      <x:c r="K57" s="23" t="str">
-        <x:v>1206.4 ms</x:v>
-      </x:c>
-      <x:c r="L57" s="23" t="str">
-        <x:v>1785.7 ms</x:v>
-      </x:c>
-      <x:c r="M57" s="23" t="str">
-        <x:v>2735.5 ms</x:v>
-      </x:c>
-      <x:c r="N57" s="23" t="str">
-        <x:v>3424.8 ms</x:v>
-      </x:c>
-      <x:c r="O57" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H57" s="27" t="n">
+        <x:v>3009.841</x:v>
+      </x:c>
+      <x:c r="I57" s="27" t="n">
+        <x:v>2623.561</x:v>
+      </x:c>
+      <x:c r="J57" s="27" t="n">
+        <x:v>1889.777</x:v>
+      </x:c>
+      <x:c r="K57" s="27"/>
+      <x:c r="L57" s="27"/>
+      <x:c r="M57" s="27"/>
+      <x:c r="N57" s="27"/>
+      <x:c r="O57" s="27"/>
       <x:c r="P57" s="27" t="n">
+        <x:v>1206.422</x:v>
+      </x:c>
+      <x:c r="Q57" s="27"/>
+      <x:c r="R57" s="27" t="n">
+        <x:v>1785.711</x:v>
+      </x:c>
+      <x:c r="S57" s="27" t="n">
+        <x:v>2735.531</x:v>
+      </x:c>
+      <x:c r="T57" s="27" t="n">
+        <x:v>3424.768</x:v>
+      </x:c>
+      <x:c r="U57" s="27"/>
+      <x:c r="V57" s="27"/>
+      <x:c r="W57" s="27"/>
+      <x:c r="X57" s="27"/>
+      <x:c r="Y57" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F57,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>16675.611</x:v>
       </x:c>
-      <x:c r="Q57" s="27" t="n">
+      <x:c r="Z57" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F57)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R57" s="23" t="str">
+      <x:c r="AA57" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5528,39 +5978,46 @@
       <x:c r="G58" s="23" t="str">
         <x:v>查询深圳梅沙湾D-HRH-2和深圳大梅沙D-HRH-1这两个5G小区的方位角和经度，筛选出方位角在90到180度之间的小区，返回小区名称、方位角和经度。</x:v>
       </x:c>
-      <x:c r="H58" s="23" t="str">
-        <x:v>3597.2 ms</x:v>
-      </x:c>
-      <x:c r="I58" s="23" t="str">
-        <x:v>2898.4 ms</x:v>
-      </x:c>
-      <x:c r="J58" s="23" t="str">
-        <x:v>2097.7 ms</x:v>
-      </x:c>
-      <x:c r="K58" s="23" t="str">
-        <x:v>1687.4 ms</x:v>
-      </x:c>
-      <x:c r="L58" s="23" t="str">
-        <x:v>2767.5 ms</x:v>
-      </x:c>
-      <x:c r="M58" s="23" t="str">
-        <x:v>3447.1 ms</x:v>
-      </x:c>
-      <x:c r="N58" s="23" t="str">
-        <x:v>3833.8 ms</x:v>
-      </x:c>
-      <x:c r="O58" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H58" s="27" t="n">
+        <x:v>3597.179</x:v>
+      </x:c>
+      <x:c r="I58" s="27" t="n">
+        <x:v>2898.41</x:v>
+      </x:c>
+      <x:c r="J58" s="27" t="n">
+        <x:v>2097.725</x:v>
+      </x:c>
+      <x:c r="K58" s="27"/>
+      <x:c r="L58" s="27"/>
+      <x:c r="M58" s="27"/>
+      <x:c r="N58" s="27"/>
+      <x:c r="O58" s="27"/>
       <x:c r="P58" s="27" t="n">
+        <x:v>1687.373</x:v>
+      </x:c>
+      <x:c r="Q58" s="27"/>
+      <x:c r="R58" s="27" t="n">
+        <x:v>2767.485</x:v>
+      </x:c>
+      <x:c r="S58" s="27" t="n">
+        <x:v>3447.067</x:v>
+      </x:c>
+      <x:c r="T58" s="27" t="n">
+        <x:v>3833.761</x:v>
+      </x:c>
+      <x:c r="U58" s="27"/>
+      <x:c r="V58" s="27"/>
+      <x:c r="W58" s="27"/>
+      <x:c r="X58" s="27"/>
+      <x:c r="Y58" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F58,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>20329</x:v>
       </x:c>
-      <x:c r="Q58" s="27" t="n">
+      <x:c r="Z58" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F58)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R58" s="23" t="str">
+      <x:c r="AA58" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5586,39 +6043,46 @@
       <x:c r="G59" s="23" t="str">
         <x:v>查询CBN-深圳梅沙湾U-H5H站点下机械下倾角等于6且电子下倾角不超过9的小区，返回小区名称、机械下倾角和电子下倾角</x:v>
       </x:c>
-      <x:c r="H59" s="23" t="str">
-        <x:v>4372.2 ms</x:v>
-      </x:c>
-      <x:c r="I59" s="23" t="str">
-        <x:v>3360.3 ms</x:v>
-      </x:c>
-      <x:c r="J59" s="23" t="str">
-        <x:v>2082.3 ms</x:v>
-      </x:c>
-      <x:c r="K59" s="23" t="str">
-        <x:v>1325.4 ms</x:v>
-      </x:c>
-      <x:c r="L59" s="23" t="str">
-        <x:v>2413.3 ms</x:v>
-      </x:c>
-      <x:c r="M59" s="23" t="str">
-        <x:v>3112.9 ms</x:v>
-      </x:c>
-      <x:c r="N59" s="23" t="str">
-        <x:v>3277.5 ms</x:v>
-      </x:c>
-      <x:c r="O59" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H59" s="27" t="n">
+        <x:v>4372.17</x:v>
+      </x:c>
+      <x:c r="I59" s="27" t="n">
+        <x:v>3360.332</x:v>
+      </x:c>
+      <x:c r="J59" s="27" t="n">
+        <x:v>2082.256</x:v>
+      </x:c>
+      <x:c r="K59" s="27"/>
+      <x:c r="L59" s="27"/>
+      <x:c r="M59" s="27"/>
+      <x:c r="N59" s="27"/>
+      <x:c r="O59" s="27"/>
       <x:c r="P59" s="27" t="n">
+        <x:v>1325.356</x:v>
+      </x:c>
+      <x:c r="Q59" s="27"/>
+      <x:c r="R59" s="27" t="n">
+        <x:v>2413.283</x:v>
+      </x:c>
+      <x:c r="S59" s="27" t="n">
+        <x:v>3112.871</x:v>
+      </x:c>
+      <x:c r="T59" s="27" t="n">
+        <x:v>3277.548</x:v>
+      </x:c>
+      <x:c r="U59" s="27"/>
+      <x:c r="V59" s="27"/>
+      <x:c r="W59" s="27"/>
+      <x:c r="X59" s="27"/>
+      <x:c r="Y59" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F59,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>19943.816</x:v>
       </x:c>
-      <x:c r="Q59" s="27" t="n">
+      <x:c r="Z59" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F59)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R59" s="23" t="str">
+      <x:c r="AA59" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5644,39 +6108,46 @@
       <x:c r="G60" s="23" t="str">
         <x:v>查询小区CBN-深圳东华风车U-H5H-0711的工程参数，如果方位角为0或180，返回它的基站标识、移动网号和方位角。</x:v>
       </x:c>
-      <x:c r="H60" s="23" t="str">
-        <x:v>2965.8 ms</x:v>
-      </x:c>
-      <x:c r="I60" s="23" t="str">
-        <x:v>2841.8 ms</x:v>
-      </x:c>
-      <x:c r="J60" s="23" t="str">
-        <x:v>2787.2 ms</x:v>
-      </x:c>
-      <x:c r="K60" s="23" t="str">
-        <x:v>1583.3 ms</x:v>
-      </x:c>
-      <x:c r="L60" s="23" t="str">
-        <x:v>1498.4 ms</x:v>
-      </x:c>
-      <x:c r="M60" s="23" t="str">
-        <x:v>3233.3 ms</x:v>
-      </x:c>
-      <x:c r="N60" s="23" t="str">
-        <x:v>3125.2 ms</x:v>
-      </x:c>
-      <x:c r="O60" s="23" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H60" s="27" t="n">
+        <x:v>2965.828</x:v>
+      </x:c>
+      <x:c r="I60" s="27" t="n">
+        <x:v>2841.778</x:v>
+      </x:c>
+      <x:c r="J60" s="27" t="n">
+        <x:v>2787.16</x:v>
+      </x:c>
+      <x:c r="K60" s="27"/>
+      <x:c r="L60" s="27"/>
+      <x:c r="M60" s="27"/>
+      <x:c r="N60" s="27"/>
+      <x:c r="O60" s="27"/>
       <x:c r="P60" s="27" t="n">
+        <x:v>1583.254</x:v>
+      </x:c>
+      <x:c r="Q60" s="27"/>
+      <x:c r="R60" s="27" t="n">
+        <x:v>1498.391</x:v>
+      </x:c>
+      <x:c r="S60" s="27" t="n">
+        <x:v>3233.27</x:v>
+      </x:c>
+      <x:c r="T60" s="27" t="n">
+        <x:v>3125.22</x:v>
+      </x:c>
+      <x:c r="U60" s="27"/>
+      <x:c r="V60" s="27"/>
+      <x:c r="W60" s="27"/>
+      <x:c r="X60" s="27"/>
+      <x:c r="Y60" s="27" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F60,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>18034.901</x:v>
       </x:c>
-      <x:c r="Q60" s="27" t="n">
+      <x:c r="Z60" s="27" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F60)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R60" s="23" t="str">
+      <x:c r="AA60" s="23" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
@@ -5702,44 +6173,51 @@
       <x:c r="G61" s="24" t="str">
         <x:v>查询站点 CBN-福州仓山-福州南站火车南站西北美化塔C-HRRH 和 CBN-深圳天麓八区U-H5H 下，天线高度不等于20米的小区，返回小区名称、天线高度和纬度。</x:v>
       </x:c>
-      <x:c r="H61" s="24" t="str">
-        <x:v>4092.0 ms</x:v>
-      </x:c>
-      <x:c r="I61" s="24" t="str">
-        <x:v>3644.6 ms</x:v>
-      </x:c>
-      <x:c r="J61" s="24" t="str">
-        <x:v>2556.4 ms</x:v>
-      </x:c>
-      <x:c r="K61" s="24" t="str">
-        <x:v>1661.0 ms</x:v>
-      </x:c>
-      <x:c r="L61" s="24" t="str">
-        <x:v>3576.4 ms</x:v>
-      </x:c>
-      <x:c r="M61" s="24" t="str">
-        <x:v>6476.4 ms</x:v>
-      </x:c>
-      <x:c r="N61" s="24" t="str">
-        <x:v>2149.3 ms</x:v>
-      </x:c>
-      <x:c r="O61" s="24" t="str">
-        <x:v>—</x:v>
-      </x:c>
+      <x:c r="H61" s="28" t="n">
+        <x:v>4091.976</x:v>
+      </x:c>
+      <x:c r="I61" s="28" t="n">
+        <x:v>3644.628</x:v>
+      </x:c>
+      <x:c r="J61" s="28" t="n">
+        <x:v>2556.391</x:v>
+      </x:c>
+      <x:c r="K61" s="28"/>
+      <x:c r="L61" s="28"/>
+      <x:c r="M61" s="28"/>
+      <x:c r="N61" s="28"/>
+      <x:c r="O61" s="28"/>
       <x:c r="P61" s="28" t="n">
+        <x:v>1660.978</x:v>
+      </x:c>
+      <x:c r="Q61" s="28"/>
+      <x:c r="R61" s="28" t="n">
+        <x:v>3576.389</x:v>
+      </x:c>
+      <x:c r="S61" s="28" t="n">
+        <x:v>6476.443</x:v>
+      </x:c>
+      <x:c r="T61" s="28" t="n">
+        <x:v>2149.299</x:v>
+      </x:c>
+      <x:c r="U61" s="28"/>
+      <x:c r="V61" s="28"/>
+      <x:c r="W61" s="28"/>
+      <x:c r="X61" s="28"/>
+      <x:c r="Y61" s="28" t="n">
         <x:f>SUMIF('调用明细'!$A$2:$A$432,F61,'调用明细'!$H$2:$H$432)</x:f>
         <x:v>24156.104</x:v>
       </x:c>
-      <x:c r="Q61" s="28" t="n">
+      <x:c r="Z61" s="28" t="n">
         <x:f>COUNTIF('调用明细'!$A$2:$A$432,F61)</x:f>
         <x:v>7</x:v>
       </x:c>
-      <x:c r="R61" s="24" t="str">
+      <x:c r="AA61" s="24" t="str">
         <x:v>完整</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
-  <x:conditionalFormatting sqref="R2:R61">
+  <x:conditionalFormatting sqref="AA2:AA61">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="缺少"/>
     <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="完整"/>
   </x:conditionalFormatting>
@@ -22631,7 +23109,7 @@
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
       <x:c r="A1" s="42" t="str">
-        <x:v>AICO Agent 模型调用时延汇总</x:v>
+        <x:v>AICO Agent 模型调用时延汇总（data1）</x:v>
       </x:c>
       <x:c r="B1" s="42"/>
       <x:c r="C1" s="42"/>
@@ -22861,150 +23339,200 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="46" t="str">
+        <x:v>AICO错误/失败</x:v>
+      </x:c>
+      <x:c r="B12" s="49" t="n">
+        <x:f>COUNTIF('调用明细'!$D$2:$D$432,A12)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C12" s="49" t="n">
+        <x:f>SUMIF('调用明细'!$D$2:$D$432,A12,'调用明细'!$H$2:$H$432)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D12" s="49" t="n">
+        <x:f>IFERROR(C12/B12,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E12" s="49" t="n">
+        <x:f>D12/1000</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="49" t="n">
+        <x:f>C12/60</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="46" t="str">
+        <x:v>未匹配/探活调用</x:v>
+      </x:c>
+      <x:c r="B13" s="49" t="n">
+        <x:f>COUNTIF('调用明细'!$D$2:$D$432,A13)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C13" s="49" t="n">
+        <x:f>SUMIF('调用明细'!$D$2:$D$432,A13,'调用明细'!$H$2:$H$432)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="D13" s="49" t="n">
+        <x:f>IFERROR(C13/B13,0)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E13" s="49" t="n">
+        <x:f>D13/1000</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F13" s="49" t="n">
+        <x:f>C13/60</x:f>
+        <x:v>0</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="46" t="str">
         <x:v>Recipe合计</x:v>
       </x:c>
-      <x:c r="B12" s="49" t="n">
+      <x:c r="B14" s="49" t="n">
         <x:f>SUM(B6:B8)</x:f>
         <x:v>187</x:v>
       </x:c>
-      <x:c r="C12" s="49" t="n">
+      <x:c r="C14" s="49" t="n">
         <x:f>SUM(C6:C8)</x:f>
         <x:v>523231.65599999996</x:v>
       </x:c>
-      <x:c r="D12" s="49" t="n">
-        <x:f>IFERROR(C12/B12,0)</x:f>
+      <x:c r="D14" s="49" t="n">
+        <x:f>IFERROR(C14/B14,0)</x:f>
         <x:v>2798.0302459893046</x:v>
       </x:c>
-      <x:c r="E12" s="49" t="n">
-        <x:f>D12/1000</x:f>
+      <x:c r="E14" s="49" t="n">
+        <x:f>D14/1000</x:f>
         <x:v>2.7980302459893047</x:v>
       </x:c>
-      <x:c r="F12" s="49" t="n">
-        <x:f>C12/60</x:f>
+      <x:c r="F14" s="49" t="n">
+        <x:f>C14/60</x:f>
         <x:v>8720.5276</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
-      <x:c r="A13" s="47" t="str">
+    <x:row r="15">
+      <x:c r="A15" s="47" t="str">
         <x:v>全部模型调用</x:v>
       </x:c>
-      <x:c r="B13" s="50" t="n">
+      <x:c r="B15" s="50" t="n">
         <x:f>COUNT('调用明细'!$H$2:$H$432)</x:f>
         <x:v>431</x:v>
       </x:c>
-      <x:c r="C13" s="50" t="n">
+      <x:c r="C15" s="50" t="n">
         <x:f>SUM('调用明细'!$H$2:$H$432)</x:f>
         <x:v>1663013.4889999994</x:v>
       </x:c>
-      <x:c r="D13" s="50" t="n">
-        <x:f>IFERROR(C13/B13,0)</x:f>
+      <x:c r="D15" s="50" t="n">
+        <x:f>IFERROR(C15/B15,0)</x:f>
         <x:v>3858.4999744779566</x:v>
       </x:c>
-      <x:c r="E13" s="50" t="n">
-        <x:f>D13/1000</x:f>
+      <x:c r="E15" s="50" t="n">
+        <x:f>D15/1000</x:f>
         <x:v>3.8584999744779567</x:v>
       </x:c>
-      <x:c r="F13" s="50" t="n">
-        <x:f>C13/60</x:f>
+      <x:c r="F15" s="50" t="n">
+        <x:f>C15/60</x:f>
         <x:v>27716.891483333322</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" s="45" t="str">
+    <x:row r="17">
+      <x:c r="A17" s="45" t="str">
         <x:v>数据质量检查</x:v>
       </x:c>
-      <x:c r="B15" s="45" t="str">
+      <x:c r="B17" s="45" t="str">
         <x:v>数量</x:v>
       </x:c>
-      <x:c r="C15" s="45" t="str">
+      <x:c r="C17" s="45" t="str">
         <x:v>说明</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="46" t="str">
-        <x:v>Excel问题数</x:v>
-      </x:c>
-      <x:c r="B16" s="51" t="n">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="C16" s="53" t="str">
-        <x:v>原表C列问题</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="46" t="str">
-        <x:v>已提取转换问题</x:v>
-      </x:c>
-      <x:c r="B17" s="51" t="n">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="C17" s="53" t="str">
-        <x:v>来自AICO Workflow/Skill参数</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="46" t="str">
-        <x:v>AICO日志行数</x:v>
+        <x:v>Excel问题数</x:v>
       </x:c>
       <x:c r="B18" s="51" t="n">
-        <x:v>185</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C18" s="53" t="str">
-        <x:v>dsv4_212_1_aico.jsonl</x:v>
+        <x:v>原表C列问题</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="46" t="str">
-        <x:v>Recipe DS日志行数</x:v>
+        <x:v>已提取转换问题</x:v>
       </x:c>
       <x:c r="B19" s="51" t="n">
-        <x:v>124</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C19" s="53" t="str">
-        <x:v>含DeepSeek与问题推荐</x:v>
+        <x:v>来自AICO Workflow/Skill参数</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="46" t="str">
-        <x:v>Qwen日志行数</x:v>
+        <x:v>AICO日志行数</x:v>
       </x:c>
       <x:c r="B20" s="51" t="n">
-        <x:v>122</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="C20" s="53" t="str">
-        <x:v>最后一次标记为Qwen总结</x:v>
+        <x:v>dsv4_212_1_aico.jsonl</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="46" t="str">
-        <x:v>未匹配调用数</x:v>
+        <x:v>Recipe DS日志行数</x:v>
       </x:c>
       <x:c r="B21" s="51" t="n">
-        <x:v>0</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="C21" s="53" t="str">
-        <x:v>需结合调用明细复核</x:v>
+        <x:v>含DeepSeek与问题推荐</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="46" t="str">
+        <x:v>Qwen日志行数</x:v>
+      </x:c>
+      <x:c r="B22" s="51" t="n">
+        <x:v>122</x:v>
+      </x:c>
+      <x:c r="C22" s="53" t="str">
+        <x:v>最后一次标记为Qwen总结</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="46" t="str">
+        <x:v>未匹配/探活调用数</x:v>
+      </x:c>
+      <x:c r="B23" s="51" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C23" s="53" t="str">
+        <x:v>未计入60题标准阶段，详见调用明细</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="46" t="str">
         <x:v>流程完整问题数</x:v>
       </x:c>
-      <x:c r="B22" s="51" t="n">
+      <x:c r="B24" s="51" t="n">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="C22" s="53" t="str">
+      <x:c r="C24" s="53" t="str">
         <x:v>具备6个标准阶段</x:v>
       </x:c>
     </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="48" t="str">
+    <x:row r="25">
+      <x:c r="A25" s="48" t="str">
         <x:v>发现的其他AICO工具</x:v>
       </x:c>
-      <x:c r="B23" s="52" t="n">
+      <x:c r="B25" s="52" t="n">
         <x:v>4</x:v>
       </x:c>
-      <x:c r="C23" s="54" t="str">
+      <x:c r="C25" s="54" t="str">
         <x:v>详见调用明细</x:v>
       </x:c>
     </x:row>

</xml_diff>